<commit_message>
Updated shocks until 2025M12
</commit_message>
<xml_diff>
--- a/VARdata.xlsx
+++ b/VARdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/drk9452_ads_northwestern_edu/Documents/Uni/LBS PhD/Research/Projects/Oil supply shocks/Repositories/OilSupplyNewsUpdate/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{E4666CA9-3A26-40FF-83AF-CBD9E073F10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{383DACD1-2472-465F-BF77-91C183A4CCEF}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{E4666CA9-3A26-40FF-83AF-CBD9E073F10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A21402BA-0A7F-436B-8A9E-0757ED017392}"/>
   <bookViews>
-    <workbookView xWindow="86280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E64FA3D6-CEF8-4D84-93AC-D7CE42D05F79}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E64FA3D6-CEF8-4D84-93AC-D7CE42D05F79}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="631">
   <si>
     <t>POIL</t>
   </si>
@@ -1911,6 +1911,24 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>2025M07</t>
+  </si>
+  <si>
+    <t>2025M08</t>
+  </si>
+  <si>
+    <t>2025M09</t>
+  </si>
+  <si>
+    <t>2025M10</t>
+  </si>
+  <si>
+    <t>2025M11</t>
+  </si>
+  <si>
+    <t>2025M12</t>
   </si>
 </sst>
 </file>
@@ -2282,7 +2300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12E1CFC8-D9C0-4308-945A-68684190B2E6}">
-  <dimension ref="A1:G619"/>
+  <dimension ref="A1:G625"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -9288,7 +9306,7 @@
         <v>65495.8</v>
       </c>
       <c r="D305">
-        <v>2211.29806813604</v>
+        <v>2211.29806813605</v>
       </c>
       <c r="E305">
         <v>81.197329999999994</v>
@@ -9380,7 +9398,7 @@
         <v>65664.25</v>
       </c>
       <c r="D309">
-        <v>2217.3170949144601</v>
+        <v>2217.3170949144501</v>
       </c>
       <c r="E309">
         <v>82.928759999999997</v>
@@ -9403,7 +9421,7 @@
         <v>65708.44</v>
       </c>
       <c r="D310">
-        <v>2203.5689150129101</v>
+        <v>2203.5689150128801</v>
       </c>
       <c r="E310">
         <v>83.467060000000004</v>
@@ -9426,7 +9444,7 @@
         <v>66214.94</v>
       </c>
       <c r="D311">
-        <v>2195.96091821457</v>
+        <v>2195.9609182145</v>
       </c>
       <c r="E311">
         <v>83.950220000000002</v>
@@ -9449,7 +9467,7 @@
         <v>66194.06</v>
       </c>
       <c r="D312">
-        <v>2183.2736513333898</v>
+        <v>2183.2736513332902</v>
       </c>
       <c r="E312">
         <v>84.743189999999998</v>
@@ -9472,7 +9490,7 @@
         <v>65383.96</v>
       </c>
       <c r="D313">
-        <v>2178.7993225515502</v>
+        <v>2178.7993225514501</v>
       </c>
       <c r="E313">
         <v>85.532560000000004</v>
@@ -9495,7 +9513,7 @@
         <v>66449.88</v>
       </c>
       <c r="D314">
-        <v>2170.8562407787599</v>
+        <v>2170.8562407787399</v>
       </c>
       <c r="E314">
         <v>85.323189999999997</v>
@@ -9518,7 +9536,7 @@
         <v>67041.63</v>
       </c>
       <c r="D315">
-        <v>2175.6147332297501</v>
+        <v>2175.6147332298801</v>
       </c>
       <c r="E315">
         <v>85.634529999999998</v>
@@ -9541,7 +9559,7 @@
         <v>67073.56</v>
       </c>
       <c r="D316">
-        <v>2156.6293973929501</v>
+        <v>2156.6293973933698</v>
       </c>
       <c r="E316">
         <v>86.065070000000006</v>
@@ -9564,7 +9582,7 @@
         <v>67735.19</v>
       </c>
       <c r="D317">
-        <v>2154.8446319209802</v>
+        <v>2154.8446319217401</v>
       </c>
       <c r="E317">
         <v>86.918080000000003</v>
@@ -9587,7 +9605,7 @@
         <v>68247.25</v>
       </c>
       <c r="D318">
-        <v>2142.4075485993599</v>
+        <v>2142.4075486001502</v>
       </c>
       <c r="E318">
         <v>87.355999999999995</v>
@@ -9610,7 +9628,7 @@
         <v>68040.13</v>
       </c>
       <c r="D319">
-        <v>2153.0586370183901</v>
+        <v>2153.0586370187002</v>
       </c>
       <c r="E319">
         <v>87.443349999999995</v>
@@ -9633,7 +9651,7 @@
         <v>68665.06</v>
       </c>
       <c r="D320">
-        <v>2157.1370711309</v>
+        <v>2157.1370711303398</v>
       </c>
       <c r="E320">
         <v>87.759680000000003</v>
@@ -9656,7 +9674,7 @@
         <v>69491.88</v>
       </c>
       <c r="D321">
-        <v>2163.1070358065099</v>
+        <v>2163.1070358050401</v>
       </c>
       <c r="E321">
         <v>88.185360000000003</v>
@@ -9679,7 +9697,7 @@
         <v>69501.440000000002</v>
       </c>
       <c r="D322">
-        <v>2165.6827358302198</v>
+        <v>2165.6827358274199</v>
       </c>
       <c r="E322">
         <v>87.989270000000005</v>
@@ -9702,7 +9720,7 @@
         <v>69945.88</v>
       </c>
       <c r="D323">
-        <v>2152.3461267586699</v>
+        <v>2152.34612675574</v>
       </c>
       <c r="E323">
         <v>88.280940000000001</v>
@@ -9725,7 +9743,7 @@
         <v>70501.31</v>
       </c>
       <c r="D324">
-        <v>2159.4386929259699</v>
+        <v>2159.4386929238399</v>
       </c>
       <c r="E324">
         <v>88.602180000000004</v>
@@ -9748,7 +9766,7 @@
         <v>69239.88</v>
       </c>
       <c r="D325">
-        <v>2180.6370177027002</v>
+        <v>2180.6370177005301</v>
       </c>
       <c r="E325">
         <v>88.918909999999997</v>
@@ -9771,7 +9789,7 @@
         <v>69158.38</v>
       </c>
       <c r="D326">
-        <v>2149.3658438428502</v>
+        <v>2149.3658438392499</v>
       </c>
       <c r="E326">
         <v>87.723500000000001</v>
@@ -9794,7 +9812,7 @@
         <v>68689.75</v>
       </c>
       <c r="D327">
-        <v>2113.80788041184</v>
+        <v>2113.8078804081301</v>
       </c>
       <c r="E327">
         <v>88.453180000000003</v>
@@ -9817,7 +9835,7 @@
         <v>69352.19</v>
       </c>
       <c r="D328">
-        <v>2154.6656920908799</v>
+        <v>2154.6656920932301</v>
       </c>
       <c r="E328">
         <v>87.630679999999998</v>
@@ -9840,7 +9858,7 @@
         <v>68419.19</v>
       </c>
       <c r="D329">
-        <v>2178.87413201249</v>
+        <v>2178.8741320292102</v>
       </c>
       <c r="E329">
         <v>87.244709999999998</v>
@@ -9863,7 +9881,7 @@
         <v>67731.94</v>
       </c>
       <c r="D330">
-        <v>2162.8974506377199</v>
+        <v>2162.8974506794598</v>
       </c>
       <c r="E330">
         <v>87.226910000000004</v>
@@ -9886,7 +9904,7 @@
         <v>66173.25</v>
       </c>
       <c r="D331">
-        <v>2117.34371879018</v>
+        <v>2117.3437188552598</v>
       </c>
       <c r="E331">
         <v>87.014679999999998</v>
@@ -9909,7 +9927,7 @@
         <v>68112.56</v>
       </c>
       <c r="D332">
-        <v>2139.7228613776601</v>
+        <v>2139.7228614330602</v>
       </c>
       <c r="E332">
         <v>86.409419999999997</v>
@@ -9932,7 +9950,7 @@
         <v>68286.63</v>
       </c>
       <c r="D333">
-        <v>2152.4458184754799</v>
+        <v>2152.4458184642799</v>
       </c>
       <c r="E333">
         <v>86.883610000000004</v>
@@ -9955,7 +9973,7 @@
         <v>67814.69</v>
       </c>
       <c r="D334">
-        <v>2158.6244139106798</v>
+        <v>2158.6244137918802</v>
       </c>
       <c r="E334">
         <v>86.290890000000005</v>
@@ -9978,7 +9996,7 @@
         <v>67716.5</v>
       </c>
       <c r="D335">
-        <v>2161.0858806292099</v>
+        <v>2161.0858804304999</v>
       </c>
       <c r="E335">
         <v>86.007919999999999</v>
@@ -10001,7 +10019,7 @@
         <v>68069.63</v>
       </c>
       <c r="D336">
-        <v>2160.5675624978799</v>
+        <v>2160.5675622494</v>
       </c>
       <c r="E336">
         <v>85.776430000000005</v>
@@ -10024,7 +10042,7 @@
         <v>67653.31</v>
       </c>
       <c r="D337">
-        <v>2172.6545008112698</v>
+        <v>2172.6545006773299</v>
       </c>
       <c r="E337">
         <v>85.842770000000002</v>
@@ -10047,7 +10065,7 @@
         <v>66803.63</v>
       </c>
       <c r="D338">
-        <v>2186.7422871202798</v>
+        <v>2186.7422872437501</v>
       </c>
       <c r="E338">
         <v>86.752880000000005</v>
@@ -10070,7 +10088,7 @@
         <v>66897.13</v>
       </c>
       <c r="D339">
-        <v>2214.7571550347002</v>
+        <v>2214.7571554569599</v>
       </c>
       <c r="E339">
         <v>86.518349999999998</v>
@@ -10093,7 +10111,7 @@
         <v>66698.44</v>
       </c>
       <c r="D340">
-        <v>2200.4284291144099</v>
+        <v>2200.4284296148699</v>
       </c>
       <c r="E340">
         <v>87.361170000000001</v>
@@ -10116,7 +10134,7 @@
         <v>66176.75</v>
       </c>
       <c r="D341">
-        <v>2170.54246124579</v>
+        <v>2170.5424615449201</v>
       </c>
       <c r="E341">
         <v>87.974559999999997</v>
@@ -10139,7 +10157,7 @@
         <v>66750.559999999998</v>
       </c>
       <c r="D342">
-        <v>2193.6417587330702</v>
+        <v>2193.6417587266101</v>
       </c>
       <c r="E342">
         <v>88.308300000000003</v>
@@ -10162,7 +10180,7 @@
         <v>66606.81</v>
       </c>
       <c r="D343">
-        <v>2203.3106104992999</v>
+        <v>2203.3106102951201</v>
       </c>
       <c r="E343">
         <v>88.481049999999996</v>
@@ -10185,7 +10203,7 @@
         <v>67068.31</v>
       </c>
       <c r="D344">
-        <v>2189.79308935176</v>
+        <v>2189.7930890934399</v>
       </c>
       <c r="E344">
         <v>88.838800000000006</v>
@@ -10208,7 +10226,7 @@
         <v>66793.75</v>
       </c>
       <c r="D345">
-        <v>2195.27730817259</v>
+        <v>2195.2773078457299</v>
       </c>
       <c r="E345">
         <v>89.144130000000004</v>
@@ -10231,7 +10249,7 @@
         <v>67330.38</v>
       </c>
       <c r="D346">
-        <v>2157.2863197848201</v>
+        <v>2157.28631922155</v>
       </c>
       <c r="E346">
         <v>89.408810000000003</v>
@@ -10254,7 +10272,7 @@
         <v>68739.25</v>
       </c>
       <c r="D347">
-        <v>2203.7725490923899</v>
+        <v>2203.7725483568202</v>
       </c>
       <c r="E347">
         <v>89.506450000000001</v>
@@ -10277,7 +10295,7 @@
         <v>68837.19</v>
       </c>
       <c r="D348">
-        <v>2207.63788907655</v>
+        <v>2207.63788825552</v>
       </c>
       <c r="E348">
         <v>89.820520000000002</v>
@@ -10300,7 +10318,7 @@
         <v>67179.81</v>
       </c>
       <c r="D349">
-        <v>2207.4986781754601</v>
+        <v>2207.4986779843898</v>
       </c>
       <c r="E349">
         <v>89.514849999999996</v>
@@ -10323,7 +10341,7 @@
         <v>67722.06</v>
       </c>
       <c r="D350">
-        <v>2220.5258495669</v>
+        <v>2220.5258507312701</v>
       </c>
       <c r="E350">
         <v>90.516170000000002</v>
@@ -10346,7 +10364,7 @@
         <v>69312.38</v>
       </c>
       <c r="D351">
-        <v>2216.0744689901799</v>
+        <v>2216.0744713572299</v>
       </c>
       <c r="E351">
         <v>90.493579999999994</v>
@@ -10369,7 +10387,7 @@
         <v>69844.63</v>
       </c>
       <c r="D352">
-        <v>2240.9053067314899</v>
+        <v>2240.9053091176202</v>
       </c>
       <c r="E352">
         <v>90.541089999999997</v>
@@ -10392,7 +10410,7 @@
         <v>68764.63</v>
       </c>
       <c r="D353">
-        <v>2242.2133335499998</v>
+        <v>2242.2133344307499</v>
       </c>
       <c r="E353">
         <v>90.274919999999995</v>
@@ -10415,7 +10433,7 @@
         <v>68761.75</v>
       </c>
       <c r="D354">
-        <v>2229.7249011119202</v>
+        <v>2229.72490001297</v>
       </c>
       <c r="E354">
         <v>90.132419999999996</v>
@@ -10438,7 +10456,7 @@
         <v>67951.81</v>
       </c>
       <c r="D355">
-        <v>2247.8630552927202</v>
+        <v>2247.8630530001201</v>
       </c>
       <c r="E355">
         <v>90.549040000000005</v>
@@ -10461,7 +10479,7 @@
         <v>68570.63</v>
       </c>
       <c r="D356">
-        <v>2273.6396889907901</v>
+        <v>2273.6396867681001</v>
       </c>
       <c r="E356">
         <v>91.219329999999999</v>
@@ -10484,7 +10502,7 @@
         <v>69025.69</v>
       </c>
       <c r="D357">
-        <v>2281.5909970559101</v>
+        <v>2281.5909954422</v>
       </c>
       <c r="E357">
         <v>91.101550000000003</v>
@@ -10507,7 +10525,7 @@
         <v>69694.31</v>
       </c>
       <c r="D358">
-        <v>2303.9354567782402</v>
+        <v>2303.9354548092001</v>
       </c>
       <c r="E358">
         <v>91.965869999999995</v>
@@ -10530,7 +10548,7 @@
         <v>70598.75</v>
       </c>
       <c r="D359">
-        <v>2302.45398373328</v>
+        <v>2302.4539815002599</v>
       </c>
       <c r="E359">
         <v>92.80256</v>
@@ -10553,7 +10571,7 @@
         <v>70831.13</v>
       </c>
       <c r="D360">
-        <v>2308.39309416572</v>
+        <v>2308.3930929426901</v>
       </c>
       <c r="E360">
         <v>93.109260000000006</v>
@@ -10576,7 +10594,7 @@
         <v>72088.19</v>
       </c>
       <c r="D361">
-        <v>2315.3839728810399</v>
+        <v>2315.3839751594101</v>
       </c>
       <c r="E361">
         <v>93.794749999999993</v>
@@ -10599,7 +10617,7 @@
         <v>71775.75</v>
       </c>
       <c r="D362">
-        <v>2319.32593780241</v>
+        <v>2319.32594417682</v>
       </c>
       <c r="E362">
         <v>93.643230000000003</v>
@@ -10622,7 +10640,7 @@
         <v>71755.13</v>
       </c>
       <c r="D363">
-        <v>2334.8587221369798</v>
+        <v>2334.85873076599</v>
       </c>
       <c r="E363">
         <v>94.864930000000001</v>
@@ -10645,7 +10663,7 @@
         <v>71699.81</v>
       </c>
       <c r="D364">
-        <v>2326.5790674855998</v>
+        <v>2326.57908435737</v>
       </c>
       <c r="E364">
         <v>94.842579999999998</v>
@@ -10668,7 +10686,7 @@
         <v>71665.88</v>
       </c>
       <c r="D365">
-        <v>2343.8832286816801</v>
+        <v>2343.8832265390602</v>
       </c>
       <c r="E365">
         <v>95.461780000000005</v>
@@ -10691,7 +10709,7 @@
         <v>71341.94</v>
       </c>
       <c r="D366">
-        <v>2353.5361234817101</v>
+        <v>2353.5361131027198</v>
       </c>
       <c r="E366">
         <v>95.780320000000003</v>
@@ -10714,7 +10732,7 @@
         <v>72940.31</v>
       </c>
       <c r="D367">
-        <v>2359.3582600847299</v>
+        <v>2359.3582335709302</v>
       </c>
       <c r="E367">
         <v>95.707149999999999</v>
@@ -10737,7 +10755,7 @@
         <v>73397.06</v>
       </c>
       <c r="D368">
-        <v>2349.97526918228</v>
+        <v>2349.9752558068099</v>
       </c>
       <c r="E368">
         <v>96.365390000000005</v>
@@ -10760,7 +10778,7 @@
         <v>72367.31</v>
       </c>
       <c r="D369">
-        <v>2322.1672968418702</v>
+        <v>2322.16729310646</v>
       </c>
       <c r="E369">
         <v>96.41619</v>
@@ -10783,7 +10801,7 @@
         <v>72987.88</v>
       </c>
       <c r="D370">
-        <v>2338.96984911754</v>
+        <v>2338.9698542686201</v>
       </c>
       <c r="E370">
         <v>96.805130000000005</v>
@@ -10806,7 +10824,7 @@
         <v>73603.19</v>
       </c>
       <c r="D371">
-        <v>2359.4495404715599</v>
+        <v>2359.4495494002499</v>
       </c>
       <c r="E371">
         <v>97.240899999999996</v>
@@ -10829,7 +10847,7 @@
         <v>73264.88</v>
       </c>
       <c r="D372">
-        <v>2395.6512507815801</v>
+        <v>2395.6512599327798</v>
       </c>
       <c r="E372">
         <v>97.384119999999996</v>
@@ -10852,7 +10870,7 @@
         <v>72898.13</v>
       </c>
       <c r="D373">
-        <v>2377.5271222522101</v>
+        <v>2377.5271348431102</v>
       </c>
       <c r="E373">
         <v>97.728980000000007</v>
@@ -10875,7 +10893,7 @@
         <v>73182.5</v>
       </c>
       <c r="D374">
-        <v>2374.0060930692698</v>
+        <v>2374.0061100610201</v>
       </c>
       <c r="E374">
         <v>98.488140000000001</v>
@@ -10898,7 +10916,7 @@
         <v>73460.88</v>
       </c>
       <c r="D375">
-        <v>2367.6335515046999</v>
+        <v>2367.6335719599401</v>
       </c>
       <c r="E375">
         <v>98.547129999999996</v>
@@ -10921,7 +10939,7 @@
         <v>73775.38</v>
       </c>
       <c r="D376">
-        <v>2398.8338402193099</v>
+        <v>2398.83387603551</v>
       </c>
       <c r="E376">
         <v>98.779730000000001</v>
@@ -10944,7 +10962,7 @@
         <v>74067.88</v>
       </c>
       <c r="D377">
-        <v>2405.0889401989498</v>
+        <v>2405.0889320256701</v>
       </c>
       <c r="E377">
         <v>99.500789999999995</v>
@@ -10967,7 +10985,7 @@
         <v>74224.69</v>
       </c>
       <c r="D378">
-        <v>2430.9918301473099</v>
+        <v>2430.9917871614798</v>
       </c>
       <c r="E378">
         <v>99.127110000000002</v>
@@ -10990,7 +11008,7 @@
         <v>73843.19</v>
       </c>
       <c r="D379">
-        <v>2412.3788473234399</v>
+        <v>2412.3787455378201</v>
       </c>
       <c r="E379">
         <v>99.791139999999999</v>
@@ -11013,7 +11031,7 @@
         <v>73684.69</v>
       </c>
       <c r="D380">
-        <v>2429.4726274015702</v>
+        <v>2429.4725827791599</v>
       </c>
       <c r="E380">
         <v>99.880129999999994</v>
@@ -11036,7 +11054,7 @@
         <v>73727.19</v>
       </c>
       <c r="D381">
-        <v>2439.5060457683098</v>
+        <v>2439.5060412606299</v>
       </c>
       <c r="E381">
         <v>100.1999</v>
@@ -11059,7 +11077,7 @@
         <v>73286</v>
       </c>
       <c r="D382">
-        <v>2448.1865950348101</v>
+        <v>2448.18663474287</v>
       </c>
       <c r="E382">
         <v>100.28400000000001</v>
@@ -11082,7 +11100,7 @@
         <v>73381.56</v>
       </c>
       <c r="D383">
-        <v>2452.5904026411499</v>
+        <v>2452.59046426536</v>
       </c>
       <c r="E383">
         <v>100.8638</v>
@@ -11105,7 +11123,7 @@
         <v>73846.38</v>
       </c>
       <c r="D384">
-        <v>2446.6011751229598</v>
+        <v>2446.6012322953502</v>
       </c>
       <c r="E384">
         <v>101.93819999999999</v>
@@ -11128,7 +11146,7 @@
         <v>74132.56</v>
       </c>
       <c r="D385">
-        <v>2455.2765654711902</v>
+        <v>2455.2766162655698</v>
       </c>
       <c r="E385">
         <v>102.6133</v>
@@ -11151,7 +11169,7 @@
         <v>73647.38</v>
       </c>
       <c r="D386">
-        <v>2429.6622394886499</v>
+        <v>2429.6622814482698</v>
       </c>
       <c r="E386">
         <v>102.4846</v>
@@ -11174,7 +11192,7 @@
         <v>73561.88</v>
       </c>
       <c r="D387">
-        <v>2451.5034188377199</v>
+        <v>2451.50344605694</v>
       </c>
       <c r="E387">
         <v>103.3763</v>
@@ -11197,7 +11215,7 @@
         <v>73414.880000000005</v>
       </c>
       <c r="D388">
-        <v>2450.9998953806398</v>
+        <v>2450.9999360153602</v>
       </c>
       <c r="E388">
         <v>103.7015</v>
@@ -11220,7 +11238,7 @@
         <v>73481</v>
       </c>
       <c r="D389">
-        <v>2456.2342751354099</v>
+        <v>2456.2342274091202</v>
       </c>
       <c r="E389">
         <v>104.1263</v>
@@ -11243,7 +11261,7 @@
         <v>73035.69</v>
       </c>
       <c r="D390">
-        <v>2450.4828189177101</v>
+        <v>2450.4826880318901</v>
       </c>
       <c r="E390">
         <v>104.83110000000001</v>
@@ -11266,7 +11284,7 @@
         <v>72932.19</v>
       </c>
       <c r="D391">
-        <v>2449.5543007298902</v>
+        <v>2449.5539408999298</v>
       </c>
       <c r="E391">
         <v>105.1742</v>
@@ -11289,7 +11307,7 @@
         <v>73961.38</v>
       </c>
       <c r="D392">
-        <v>2460.0101003126401</v>
+        <v>2460.0100358405598</v>
       </c>
       <c r="E392">
         <v>105.5162</v>
@@ -11312,7 +11330,7 @@
         <v>73654.25</v>
       </c>
       <c r="D393">
-        <v>2461.94373831248</v>
+        <v>2461.9437661604402</v>
       </c>
       <c r="E393">
         <v>105.93040000000001</v>
@@ -11335,7 +11353,7 @@
         <v>73365.13</v>
       </c>
       <c r="D394">
-        <v>2464.47431761493</v>
+        <v>2464.4744165145498</v>
       </c>
       <c r="E394">
         <v>106.3349</v>
@@ -11358,7 +11376,7 @@
         <v>73705.81</v>
       </c>
       <c r="D395">
-        <v>2478.5094648264799</v>
+        <v>2478.5099645486098</v>
       </c>
       <c r="E395">
         <v>106.608</v>
@@ -11381,7 +11399,7 @@
         <v>73337.25</v>
       </c>
       <c r="D396">
-        <v>2496.5263264015098</v>
+        <v>2496.5263997421298</v>
       </c>
       <c r="E396">
         <v>107.87860000000001</v>
@@ -11404,7 +11422,7 @@
         <v>73117.440000000002</v>
       </c>
       <c r="D397">
-        <v>2461.2337552366198</v>
+        <v>2461.23379547594</v>
       </c>
       <c r="E397">
         <v>108.57129999999999</v>
@@ -11427,7 +11445,7 @@
         <v>72767.31</v>
       </c>
       <c r="D398">
-        <v>2462.0737234665098</v>
+        <v>2462.0737481338901</v>
       </c>
       <c r="E398">
         <v>109.2043</v>
@@ -11450,7 +11468,7 @@
         <v>73023.44</v>
       </c>
       <c r="D399">
-        <v>2475.1729666184701</v>
+        <v>2475.1729695165</v>
       </c>
       <c r="E399">
         <v>109.4357</v>
@@ -11473,7 +11491,7 @@
         <v>72945.94</v>
       </c>
       <c r="D400">
-        <v>2458.1419895650201</v>
+        <v>2458.1419686204499</v>
       </c>
       <c r="E400">
         <v>110.15179999999999</v>
@@ -11496,7 +11514,7 @@
         <v>73183.56</v>
       </c>
       <c r="D401">
-        <v>2465.3751845942602</v>
+        <v>2465.3750181661699</v>
       </c>
       <c r="E401">
         <v>110.30110000000001</v>
@@ -11519,7 +11537,7 @@
         <v>72711</v>
       </c>
       <c r="D402">
-        <v>2493.4787165461698</v>
+        <v>2493.47837597436</v>
       </c>
       <c r="E402">
         <v>111.31270000000001</v>
@@ -11542,7 +11560,7 @@
         <v>72322.44</v>
       </c>
       <c r="D403">
-        <v>2499.8049159755501</v>
+        <v>2499.8042190176702</v>
       </c>
       <c r="E403">
         <v>111.4787</v>
@@ -11565,7 +11583,7 @@
         <v>72832.13</v>
       </c>
       <c r="D404">
-        <v>2484.8247252612</v>
+        <v>2484.8246372942399</v>
       </c>
       <c r="E404">
         <v>111.97799999999999</v>
@@ -11588,7 +11606,7 @@
         <v>72184.5</v>
       </c>
       <c r="D405">
-        <v>2467.458818906</v>
+        <v>2467.4589474690601</v>
       </c>
       <c r="E405">
         <v>112.4597</v>
@@ -11611,7 +11629,7 @@
         <v>72961.38</v>
       </c>
       <c r="D406">
-        <v>2461.8476261963801</v>
+        <v>2461.8478611237601</v>
       </c>
       <c r="E406">
         <v>112.5314</v>
@@ -11634,7 +11652,7 @@
         <v>73638.5</v>
       </c>
       <c r="D407">
-        <v>2439.0794098128599</v>
+        <v>2439.0808406302199</v>
       </c>
       <c r="E407">
         <v>113.2724</v>
@@ -11657,7 +11675,7 @@
         <v>73345.81</v>
       </c>
       <c r="D408">
-        <v>2430.27080307292</v>
+        <v>2430.2708286769398</v>
       </c>
       <c r="E408">
         <v>113.74290000000001</v>
@@ -11680,7 +11698,7 @@
         <v>73789.81</v>
       </c>
       <c r="D409">
-        <v>2446.9522529075798</v>
+        <v>2446.9521726503499</v>
       </c>
       <c r="E409">
         <v>113.9851</v>
@@ -11703,7 +11721,7 @@
         <v>73874.13</v>
       </c>
       <c r="D410">
-        <v>2449.68766315117</v>
+        <v>2449.6875876582699</v>
       </c>
       <c r="E410">
         <v>115.6785</v>
@@ -11726,7 +11744,7 @@
         <v>74057.88</v>
       </c>
       <c r="D411">
-        <v>2433.8796717013402</v>
+        <v>2433.8796380693898</v>
       </c>
       <c r="E411">
         <v>115.05029999999999</v>
@@ -11749,7 +11767,7 @@
         <v>74237.88</v>
       </c>
       <c r="D412">
-        <v>2471.8949937062098</v>
+        <v>2471.8948166566402</v>
       </c>
       <c r="E412">
         <v>114.6896</v>
@@ -11772,7 +11790,7 @@
         <v>73646.13</v>
       </c>
       <c r="D413">
-        <v>2450.0978689233302</v>
+        <v>2450.0974405260399</v>
       </c>
       <c r="E413">
         <v>115.1825</v>
@@ -11795,7 +11813,7 @@
         <v>73963.44</v>
       </c>
       <c r="D414">
-        <v>2435.4748812840398</v>
+        <v>2435.4743408917702</v>
       </c>
       <c r="E414">
         <v>114.1686</v>
@@ -11818,7 +11836,7 @@
         <v>73982.94</v>
       </c>
       <c r="D415">
-        <v>2432.2548861127202</v>
+        <v>2432.2538318546999</v>
       </c>
       <c r="E415">
         <v>114.4692</v>
@@ -11841,7 +11859,7 @@
         <v>74729</v>
       </c>
       <c r="D416">
-        <v>2464.8933272348299</v>
+        <v>2464.8929037032499</v>
       </c>
       <c r="E416">
         <v>113.70659999999999</v>
@@ -11864,7 +11882,7 @@
         <v>73531.75</v>
       </c>
       <c r="D417">
-        <v>2479.36522697086</v>
+        <v>2479.3648170033898</v>
       </c>
       <c r="E417">
         <v>112.6833</v>
@@ -11887,7 +11905,7 @@
         <v>72525.5</v>
       </c>
       <c r="D418">
-        <v>2489.9600701417298</v>
+        <v>2489.9626028247799</v>
       </c>
       <c r="E418">
         <v>111.54130000000001</v>
@@ -11910,7 +11928,7 @@
         <v>73586.75</v>
       </c>
       <c r="D419">
-        <v>2498.4188147638301</v>
+        <v>2498.4204337624501</v>
       </c>
       <c r="E419">
         <v>109.8184</v>
@@ -11933,7 +11951,7 @@
         <v>73427.56</v>
       </c>
       <c r="D420">
-        <v>2505.1188271963201</v>
+        <v>2505.1183624312798</v>
       </c>
       <c r="E420">
         <v>106.8489</v>
@@ -11956,7 +11974,7 @@
         <v>72631.63</v>
       </c>
       <c r="D421">
-        <v>2523.6461133292701</v>
+        <v>2523.6458284939899</v>
       </c>
       <c r="E421">
         <v>103.4164</v>
@@ -11979,7 +11997,7 @@
         <v>71529.25</v>
       </c>
       <c r="D422">
-        <v>2535.4603557296</v>
+        <v>2535.4603304556099</v>
       </c>
       <c r="E422">
         <v>100.49039999999999</v>
@@ -12002,7 +12020,7 @@
         <v>72050.559999999998</v>
       </c>
       <c r="D423">
-        <v>2531.9336463773402</v>
+        <v>2531.9339284892999</v>
       </c>
       <c r="E423">
         <v>101.3404</v>
@@ -12025,7 +12043,7 @@
         <v>71852</v>
       </c>
       <c r="D424">
-        <v>2525.6764421552002</v>
+        <v>2525.6764987443298</v>
       </c>
       <c r="E424">
         <v>100.8404</v>
@@ -12048,7 +12066,7 @@
         <v>72003.81</v>
       </c>
       <c r="D425">
-        <v>2518.4951797403201</v>
+        <v>2518.4947360469901</v>
       </c>
       <c r="E425">
         <v>101.0283</v>
@@ -12071,7 +12089,7 @@
         <v>71594.06</v>
       </c>
       <c r="D426">
-        <v>2503.9495204465902</v>
+        <v>2503.9483545476101</v>
       </c>
       <c r="E426">
         <v>101.6028</v>
@@ -12094,7 +12112,7 @@
         <v>71796.75</v>
       </c>
       <c r="D427">
-        <v>2488.77573357437</v>
+        <v>2488.77330359706</v>
       </c>
       <c r="E427">
         <v>102.5956</v>
@@ -12117,7 +12135,7 @@
         <v>72644.38</v>
       </c>
       <c r="D428">
-        <v>2504.1734226526601</v>
+        <v>2504.1713645762402</v>
       </c>
       <c r="E428">
         <v>103.5034</v>
@@ -12140,7 +12158,7 @@
         <v>72132</v>
       </c>
       <c r="D429">
-        <v>2513.5743995657799</v>
+        <v>2513.5729187462098</v>
       </c>
       <c r="E429">
         <v>104.3562</v>
@@ -12163,7 +12181,7 @@
         <v>72612.63</v>
       </c>
       <c r="D430">
-        <v>2516.1033496835798</v>
+        <v>2516.1088831289899</v>
       </c>
       <c r="E430">
         <v>105.5352</v>
@@ -12186,7 +12204,7 @@
         <v>73068.25</v>
       </c>
       <c r="D431">
-        <v>2505.8755132610199</v>
+        <v>2505.8786106646698</v>
       </c>
       <c r="E431">
         <v>106.04770000000001</v>
@@ -12209,7 +12227,7 @@
         <v>73045.19</v>
       </c>
       <c r="D432">
-        <v>2535.6818909603899</v>
+        <v>2535.6831487220802</v>
       </c>
       <c r="E432">
         <v>107.0355</v>
@@ -12232,7 +12250,7 @@
         <v>72743.63</v>
       </c>
       <c r="D433">
-        <v>2530.3447052455799</v>
+        <v>2530.3457239131699</v>
       </c>
       <c r="E433">
         <v>107.667</v>
@@ -12255,7 +12273,7 @@
         <v>72907.25</v>
       </c>
       <c r="D434">
-        <v>2538.1596475179399</v>
+        <v>2538.1596676716799</v>
       </c>
       <c r="E434">
         <v>109.66849999999999</v>
@@ -12278,7 +12296,7 @@
         <v>73473.19</v>
       </c>
       <c r="D435">
-        <v>2528.4597957322499</v>
+        <v>2528.4589114055002</v>
       </c>
       <c r="E435">
         <v>109.52509999999999</v>
@@ -12301,7 +12319,7 @@
         <v>73774.5</v>
       </c>
       <c r="D436">
-        <v>2531.5195833521202</v>
+        <v>2531.5178021340998</v>
       </c>
       <c r="E436">
         <v>111.12949999999999</v>
@@ -12324,7 +12342,7 @@
         <v>73761.06</v>
       </c>
       <c r="D437">
-        <v>2520.94147184146</v>
+        <v>2520.9392746233002</v>
       </c>
       <c r="E437">
         <v>111.63500000000001</v>
@@ -12347,7 +12365,7 @@
         <v>73823.69</v>
       </c>
       <c r="D438">
-        <v>2526.9770167015699</v>
+        <v>2526.9743982549098</v>
       </c>
       <c r="E438">
         <v>112.58069999999999</v>
@@ -12370,7 +12388,7 @@
         <v>73935.13</v>
       </c>
       <c r="D439">
-        <v>2539.97366445132</v>
+        <v>2539.9696014074698</v>
       </c>
       <c r="E439">
         <v>112.3613</v>
@@ -12393,7 +12411,7 @@
         <v>74200</v>
       </c>
       <c r="D440">
-        <v>2531.54833113521</v>
+        <v>2531.54459989616</v>
       </c>
       <c r="E440">
         <v>112.8854</v>
@@ -12416,7 +12434,7 @@
         <v>74133.63</v>
       </c>
       <c r="D441">
-        <v>2547.6350036870699</v>
+        <v>2547.6328391881302</v>
       </c>
       <c r="E441">
         <v>113.30880000000001</v>
@@ -12439,7 +12457,7 @@
         <v>74439.88</v>
       </c>
       <c r="D442">
-        <v>2538.96693531249</v>
+        <v>2538.97705644092</v>
       </c>
       <c r="E442">
         <v>113.5702</v>
@@ -12462,7 +12480,7 @@
         <v>74332.44</v>
       </c>
       <c r="D443">
-        <v>2570.6301536669898</v>
+        <v>2570.63679950193</v>
       </c>
       <c r="E443">
         <v>114.1142</v>
@@ -12485,7 +12503,7 @@
         <v>74940</v>
       </c>
       <c r="D444">
-        <v>2543.5380050510198</v>
+        <v>2543.54426834573</v>
       </c>
       <c r="E444">
         <v>114.7718</v>
@@ -12508,7 +12526,7 @@
         <v>74893.56</v>
       </c>
       <c r="D445">
-        <v>2532.1484390110099</v>
+        <v>2532.1526665532801</v>
       </c>
       <c r="E445">
         <v>116.1199</v>
@@ -12531,7 +12549,7 @@
         <v>75386.5</v>
       </c>
       <c r="D446">
-        <v>2535.1336269816402</v>
+        <v>2535.1333467141899</v>
       </c>
       <c r="E446">
         <v>117.7303</v>
@@ -12554,7 +12572,7 @@
         <v>75141.63</v>
       </c>
       <c r="D447">
-        <v>2527.8035046104701</v>
+        <v>2527.7989571551898</v>
       </c>
       <c r="E447">
         <v>117.5355</v>
@@ -12577,7 +12595,7 @@
         <v>74122.19</v>
       </c>
       <c r="D448">
-        <v>2527.1157873912498</v>
+        <v>2527.1075486259101</v>
       </c>
       <c r="E448">
         <v>117.1961</v>
@@ -12600,7 +12618,7 @@
         <v>74059.56</v>
       </c>
       <c r="D449">
-        <v>2534.81411656609</v>
+        <v>2534.80656517236</v>
       </c>
       <c r="E449">
         <v>116.61060000000001</v>
@@ -12623,7 +12641,7 @@
         <v>73314.44</v>
       </c>
       <c r="D450">
-        <v>2531.09981822174</v>
+        <v>2531.0966973529498</v>
       </c>
       <c r="E450">
         <v>117.684</v>
@@ -12646,7 +12664,7 @@
         <v>74098.5</v>
       </c>
       <c r="D451">
-        <v>2516.7807771584398</v>
+        <v>2516.7819850849</v>
       </c>
       <c r="E451">
         <v>117.9905</v>
@@ -12669,7 +12687,7 @@
         <v>74385.88</v>
       </c>
       <c r="D452">
-        <v>2493.8360857185398</v>
+        <v>2493.8152045883298</v>
       </c>
       <c r="E452">
         <v>118.34990000000001</v>
@@ -12692,7 +12710,7 @@
         <v>74908.75</v>
       </c>
       <c r="D453">
-        <v>2465.0720776647299</v>
+        <v>2465.0733650439802</v>
       </c>
       <c r="E453">
         <v>118.6061</v>
@@ -12715,7 +12733,7 @@
         <v>74257.13</v>
       </c>
       <c r="D454">
-        <v>2439.0274498973299</v>
+        <v>2439.04148411811</v>
       </c>
       <c r="E454">
         <v>118.533</v>
@@ -12738,7 +12756,7 @@
         <v>74798.5</v>
       </c>
       <c r="D455">
-        <v>2443.6540575303902</v>
+        <v>2443.6808366294599</v>
       </c>
       <c r="E455">
         <v>118.5491</v>
@@ -12761,7 +12779,7 @@
         <v>75782.19</v>
       </c>
       <c r="D456">
-        <v>2448.9626706930298</v>
+        <v>2448.9736733670302</v>
       </c>
       <c r="E456">
         <v>118.14075730506754</v>
@@ -12784,7 +12802,7 @@
         <v>76191.81</v>
       </c>
       <c r="D457">
-        <v>2455.5739880793399</v>
+        <v>2455.58485076335</v>
       </c>
       <c r="E457">
         <v>118.41470415791355</v>
@@ -12807,7 +12825,7 @@
         <v>76337.5</v>
       </c>
       <c r="D458">
-        <v>2440.8445670226802</v>
+        <v>2440.85189403817</v>
       </c>
       <c r="E458">
         <v>119.33437715532203</v>
@@ -12830,7 +12848,7 @@
         <v>76656.06</v>
       </c>
       <c r="D459">
-        <v>2430.38548322112</v>
+        <v>2430.3894433054202</v>
       </c>
       <c r="E459">
         <v>119.58573725959694</v>
@@ -12853,7 +12871,7 @@
         <v>76340.25</v>
       </c>
       <c r="D460">
-        <v>2452.1782432939599</v>
+        <v>2452.1061064332998</v>
       </c>
       <c r="E460">
         <v>118.99054109179259</v>
@@ -12876,7 +12894,7 @@
         <v>76644.5</v>
       </c>
       <c r="D461">
-        <v>2477.4568970402502</v>
+        <v>2477.4557643661501</v>
       </c>
       <c r="E461">
         <v>118.15970701999298</v>
@@ -12899,7 +12917,7 @@
         <v>75932.94</v>
       </c>
       <c r="D462">
-        <v>2494.3610849023598</v>
+        <v>2494.3588957591701</v>
       </c>
       <c r="E462">
         <v>118.86664944643007</v>
@@ -12922,7 +12940,7 @@
         <v>75746.94</v>
       </c>
       <c r="D463">
-        <v>2504.8666116040399</v>
+        <v>2504.86511587519</v>
       </c>
       <c r="E463">
         <v>118.3926607642689</v>
@@ -12945,7 +12963,7 @@
         <v>75942.19</v>
       </c>
       <c r="D464">
-        <v>2511.6258458327802</v>
+        <v>2511.61533246917</v>
       </c>
       <c r="E464">
         <v>118.52036283139523</v>
@@ -12968,7 +12986,7 @@
         <v>75993.38</v>
       </c>
       <c r="D465">
-        <v>2515.5176308221899</v>
+        <v>2515.5184086997301</v>
       </c>
       <c r="E465">
         <v>118.16673072549602</v>
@@ -12991,7 +13009,7 @@
         <v>75481.56</v>
       </c>
       <c r="D466">
-        <v>2522.1869030602302</v>
+        <v>2522.20498781059</v>
       </c>
       <c r="E466">
         <v>117.75755242288895</v>
@@ -13014,7 +13032,7 @@
         <v>75985.31</v>
       </c>
       <c r="D467">
-        <v>2509.5553056929102</v>
+        <v>2509.60468244096</v>
       </c>
       <c r="E467">
         <v>118.35596815169392</v>
@@ -13037,7 +13055,7 @@
         <v>76528.56</v>
       </c>
       <c r="D468">
-        <v>2517.39438043057</v>
+        <v>2517.41459779977</v>
       </c>
       <c r="E468">
         <v>118.19566799799401</v>
@@ -13060,7 +13078,7 @@
         <v>76566.63</v>
       </c>
       <c r="D469">
-        <v>2500.5242694070098</v>
+        <v>2500.5429887425898</v>
       </c>
       <c r="E469">
         <v>118.57286011270736</v>
@@ -13083,7 +13101,7 @@
         <v>75888</v>
       </c>
       <c r="D470">
-        <v>2504.1677697730702</v>
+        <v>2504.1810923264602</v>
       </c>
       <c r="E470">
         <v>119.04896745594699</v>
@@ -13106,7 +13124,7 @@
         <v>75679.63</v>
       </c>
       <c r="D471">
-        <v>2507.2584525689299</v>
+        <v>2507.26629865823</v>
       </c>
       <c r="E471">
         <v>119.02866143345256</v>
@@ -13129,7 +13147,7 @@
         <v>75817.440000000002</v>
       </c>
       <c r="D472">
-        <v>2511.23787077425</v>
+        <v>2511.0954690497301</v>
       </c>
       <c r="E472">
         <v>119.35038495946846</v>
@@ -13152,7 +13170,7 @@
         <v>76247.63</v>
       </c>
       <c r="D473">
-        <v>2497.1058934092598</v>
+        <v>2497.1062753995502</v>
       </c>
       <c r="E473">
         <v>119.80717869674264</v>
@@ -13175,7 +13193,7 @@
         <v>76199.13</v>
       </c>
       <c r="D474">
-        <v>2475.7839050167199</v>
+        <v>2475.7788022517002</v>
       </c>
       <c r="E474">
         <v>119.89250139482283</v>
@@ -13198,7 +13216,7 @@
         <v>76174.25</v>
       </c>
       <c r="D475">
-        <v>2473.4341966915299</v>
+        <v>2473.4296399662599</v>
       </c>
       <c r="E475">
         <v>119.38053640623478</v>
@@ -13221,7 +13239,7 @@
         <v>76665.5</v>
       </c>
       <c r="D476">
-        <v>2487.0444901757701</v>
+        <v>2487.0511198716299</v>
       </c>
       <c r="E476">
         <v>120.06179493641287</v>
@@ -13244,7 +13262,7 @@
         <v>76426.94</v>
       </c>
       <c r="D477">
-        <v>2487.1451878002699</v>
+        <v>2487.1518459654199</v>
       </c>
       <c r="E477">
         <v>120.62158187704878</v>
@@ -13267,7 +13285,7 @@
         <v>75902.25</v>
       </c>
       <c r="D478">
-        <v>2515.5806474353599</v>
+        <v>2515.5975488243098</v>
       </c>
       <c r="E478">
         <v>120.99892306608187</v>
@@ -13290,7 +13308,7 @@
         <v>76260.88</v>
       </c>
       <c r="D479">
-        <v>2521.4655656445898</v>
+        <v>2521.5234977718501</v>
       </c>
       <c r="E479">
         <v>120.81653939296628</v>
@@ -13313,7 +13331,7 @@
         <v>76543.38</v>
       </c>
       <c r="D480">
-        <v>2516.6772533199101</v>
+        <v>2516.7565046681798</v>
       </c>
       <c r="E480">
         <v>121.39299775045774</v>
@@ -13336,7 +13354,7 @@
         <v>76886.63</v>
       </c>
       <c r="D481">
-        <v>2513.1467104118401</v>
+        <v>2513.1548951551599</v>
       </c>
       <c r="E481">
         <v>121.2350712992764</v>
@@ -13359,7 +13377,7 @@
         <v>77257.88</v>
       </c>
       <c r="D482">
-        <v>2515.6840748285099</v>
+        <v>2515.6948508032001</v>
       </c>
       <c r="E482">
         <v>122.29477842314841</v>
@@ -13382,7 +13400,7 @@
         <v>77761.56</v>
       </c>
       <c r="D483">
-        <v>2505.3316546557799</v>
+        <v>2505.3410138282502</v>
       </c>
       <c r="E483">
         <v>122.99393056930916</v>
@@ -13405,7 +13423,7 @@
         <v>77179.94</v>
       </c>
       <c r="D484">
-        <v>2502.2757895590498</v>
+        <v>2502.0569118840499</v>
       </c>
       <c r="E484">
         <v>122.80862122821897</v>
@@ -13428,7 +13446,7 @@
         <v>77247</v>
       </c>
       <c r="D485">
-        <v>2483.5576453284002</v>
+        <v>2483.5565282910402</v>
       </c>
       <c r="E485">
         <v>123.28358667038096</v>
@@ -13451,7 +13469,7 @@
         <v>76948.25</v>
       </c>
       <c r="D486">
-        <v>2490.9397997357601</v>
+        <v>2490.9273788485998</v>
       </c>
       <c r="E486">
         <v>122.99587285905162</v>
@@ -13474,7 +13492,7 @@
         <v>77353.5</v>
       </c>
       <c r="D487">
-        <v>2486.4227194835198</v>
+        <v>2486.4018912576398</v>
       </c>
       <c r="E487">
         <v>123.2257264918003</v>
@@ -13497,7 +13515,7 @@
         <v>77616.63</v>
       </c>
       <c r="D488">
-        <v>2477.1719944199599</v>
+        <v>2477.19528640931</v>
       </c>
       <c r="E488">
         <v>123.45360970387436</v>
@@ -13520,7 +13538,7 @@
         <v>77782.75</v>
       </c>
       <c r="D489">
-        <v>2493.1775937126199</v>
+        <v>2493.2375696792401</v>
       </c>
       <c r="E489">
         <v>122.25831169856602</v>
@@ -13543,7 +13561,7 @@
         <v>78668</v>
       </c>
       <c r="D490">
-        <v>2493.03028496771</v>
+        <v>2493.0531848116698</v>
       </c>
       <c r="E490">
         <v>123.48572963177847</v>
@@ -13566,7 +13584,7 @@
         <v>79410.69</v>
       </c>
       <c r="D491">
-        <v>2505.8890126103101</v>
+        <v>2505.9305361810498</v>
       </c>
       <c r="E491">
         <v>122.65342657538569</v>
@@ -13589,7 +13607,7 @@
         <v>79498.94</v>
       </c>
       <c r="D492">
-        <v>2491.9582883191001</v>
+        <v>2492.0968079374002</v>
       </c>
       <c r="E492">
         <v>123.5449340741413</v>
@@ -13612,7 +13630,7 @@
         <v>80310.25</v>
       </c>
       <c r="D493">
-        <v>2502.8254314787</v>
+        <v>2502.8193622475001</v>
       </c>
       <c r="E493">
         <v>123.82562279424961</v>
@@ -13635,7 +13653,7 @@
         <v>79728.56</v>
       </c>
       <c r="D494">
-        <v>2510.1863625527499</v>
+        <v>2510.17930661941</v>
       </c>
       <c r="E494">
         <v>124.51339629768127</v>
@@ -13658,7 +13676,7 @@
         <v>79522.880000000005</v>
       </c>
       <c r="D495">
-        <v>2534.3901514475901</v>
+        <v>2534.3801913165698</v>
       </c>
       <c r="E495">
         <v>124.17704048680501</v>
@@ -13681,7 +13699,7 @@
         <v>80422.31</v>
       </c>
       <c r="D496">
-        <v>2572.1255448685502</v>
+        <v>2571.8828599016301</v>
       </c>
       <c r="E496">
         <v>124.13239125563145</v>
@@ -13704,7 +13722,7 @@
         <v>80016.81</v>
       </c>
       <c r="D497">
-        <v>2572.32153799042</v>
+        <v>2572.3045627950901</v>
       </c>
       <c r="E497">
         <v>124.06245844535665</v>
@@ -13727,7 +13745,7 @@
         <v>79975.75</v>
       </c>
       <c r="D498">
-        <v>2586.7654751374798</v>
+        <v>2586.7429430899101</v>
       </c>
       <c r="E498">
         <v>123.74836754574204</v>
@@ -13750,7 +13768,7 @@
         <v>80397.81</v>
       </c>
       <c r="D499">
-        <v>2586.5946184457498</v>
+        <v>2586.5667089093399</v>
       </c>
       <c r="E499">
         <v>124.33509119711461</v>
@@ -13773,7 +13791,7 @@
         <v>80923.75</v>
       </c>
       <c r="D500">
-        <v>2582.9298077240401</v>
+        <v>2582.9460709750001</v>
       </c>
       <c r="E500">
         <v>124.07425868463432</v>
@@ -13796,7 +13814,7 @@
         <v>80772</v>
       </c>
       <c r="D501">
-        <v>2610.4336934888902</v>
+        <v>2610.5583441157901</v>
       </c>
       <c r="E501">
         <v>124.49109553380849</v>
@@ -13819,7 +13837,7 @@
         <v>80558.94</v>
       </c>
       <c r="D502">
-        <v>2622.9495049642301</v>
+        <v>2622.9852929798299</v>
       </c>
       <c r="E502">
         <v>124.37144851537983</v>
@@ -13842,7 +13860,7 @@
         <v>80698.75</v>
       </c>
       <c r="D503">
-        <v>2642.3287087280601</v>
+        <v>2642.3586915317001</v>
       </c>
       <c r="E503">
         <v>124.77885124480906</v>
@@ -13865,7 +13883,7 @@
         <v>81290.69</v>
       </c>
       <c r="D504">
-        <v>2650.0556516100701</v>
+        <v>2650.2511718617002</v>
       </c>
       <c r="E504">
         <v>124.31098861255964</v>
@@ -13888,7 +13906,7 @@
         <v>81446.44</v>
       </c>
       <c r="D505">
-        <v>2675.5896931602801</v>
+        <v>2675.5639957119201</v>
       </c>
       <c r="E505">
         <v>124.01275898947097</v>
@@ -13911,7 +13929,7 @@
         <v>81466.63</v>
       </c>
       <c r="D506">
-        <v>2677.0151465428498</v>
+        <v>2676.9830076767498</v>
       </c>
       <c r="E506">
         <v>125.35768452359675</v>
@@ -13934,7 +13952,7 @@
         <v>80705.06</v>
       </c>
       <c r="D507">
-        <v>2685.93895243115</v>
+        <v>2685.9051147370501</v>
       </c>
       <c r="E507">
         <v>125.02797942597637</v>
@@ -13957,7 +13975,7 @@
         <v>80676.75</v>
       </c>
       <c r="D508">
-        <v>2686.8599997421402</v>
+        <v>2686.59492505559</v>
       </c>
       <c r="E508">
         <v>125.28072428385592</v>
@@ -13980,7 +13998,7 @@
         <v>79778.25</v>
       </c>
       <c r="D509">
-        <v>2680.7035277290902</v>
+        <v>2680.6727594434401</v>
       </c>
       <c r="E509">
         <v>125.51082522869189</v>
@@ -14003,7 +14021,7 @@
         <v>78990.94</v>
       </c>
       <c r="D510">
-        <v>2693.6162826080599</v>
+        <v>2693.5809952422901</v>
       </c>
       <c r="E510">
         <v>125.44819974466931</v>
@@ -14026,7 +14044,7 @@
         <v>79889.38</v>
       </c>
       <c r="D511">
-        <v>2705.5910546789901</v>
+        <v>2705.5449003898502</v>
       </c>
       <c r="E511">
         <v>126.31682558927686</v>
@@ -14049,7 +14067,7 @@
         <v>80607.5</v>
       </c>
       <c r="D512">
-        <v>2715.7049214552599</v>
+        <v>2715.7194472967199</v>
       </c>
       <c r="E512">
         <v>125.70197635861378</v>
@@ -14072,7 +14090,7 @@
         <v>80064</v>
       </c>
       <c r="D513">
-        <v>2709.4002467238702</v>
+        <v>2709.59508099614</v>
       </c>
       <c r="E513">
         <v>126.07324989916349</v>
@@ -14095,7 +14113,7 @@
         <v>80392.06</v>
       </c>
       <c r="D514">
-        <v>2697.2775157945598</v>
+        <v>2697.3614612359802</v>
       </c>
       <c r="E514">
         <v>125.96148503155078</v>
@@ -14118,7 +14136,7 @@
         <v>81571.56</v>
       </c>
       <c r="D515">
-        <v>2698.5899174340602</v>
+        <v>2698.6320847182101</v>
       </c>
       <c r="E515">
         <v>126.83403785871297</v>
@@ -14141,7 +14159,7 @@
         <v>82631.94</v>
       </c>
       <c r="D516">
-        <v>2695.4770284206602</v>
+        <v>2695.6992901113399</v>
       </c>
       <c r="E516">
         <v>126.92318194808253</v>
@@ -14164,7 +14182,7 @@
         <v>82090.5</v>
       </c>
       <c r="D517">
-        <v>2707.02510630291</v>
+        <v>2707.0125298018102</v>
       </c>
       <c r="E517">
         <v>126.88902479694869</v>
@@ -14187,7 +14205,7 @@
         <v>81167.63</v>
       </c>
       <c r="D518">
-        <v>2730.3461344755001</v>
+        <v>2730.3526369413298</v>
       </c>
       <c r="E518">
         <v>127.85577746216126</v>
@@ -14210,7 +14228,7 @@
         <v>81183.13</v>
       </c>
       <c r="D519">
-        <v>2736.0811327758802</v>
+        <v>2735.7342897383801</v>
       </c>
       <c r="E519">
         <v>128.33369493686936</v>
@@ -14233,7 +14251,7 @@
         <v>80376.44</v>
       </c>
       <c r="D520">
-        <v>2749.6418742440901</v>
+        <v>2749.4876489220001</v>
       </c>
       <c r="E520">
         <v>129.01558161615276</v>
@@ -14256,7 +14274,7 @@
         <v>79942</v>
       </c>
       <c r="D521">
-        <v>2713.62296077887</v>
+        <v>2713.5888757610101</v>
       </c>
       <c r="E521">
         <v>129.27656943628483</v>
@@ -14279,7 +14297,7 @@
         <v>80525.19</v>
       </c>
       <c r="D522">
-        <v>2691.3278553141599</v>
+        <v>2691.3025363196898</v>
       </c>
       <c r="E522">
         <v>129.50706446858402</v>
@@ -14302,7 +14320,7 @@
         <v>81074.69</v>
       </c>
       <c r="D523">
-        <v>2687.4714631935499</v>
+        <v>2687.3763876419998</v>
       </c>
       <c r="E523">
         <v>129.47927127320767</v>
@@ -14325,7 +14343,7 @@
         <v>81591.38</v>
       </c>
       <c r="D524">
-        <v>2678.3431857834698</v>
+        <v>2678.3840965890499</v>
       </c>
       <c r="E524">
         <v>129.33671267722045</v>
@@ -14348,7 +14366,7 @@
         <v>80980.19</v>
       </c>
       <c r="D525">
-        <v>2645.32939607242</v>
+        <v>2645.5822588013498</v>
       </c>
       <c r="E525">
         <v>130.17848438081424</v>
@@ -14371,7 +14389,7 @@
         <v>81190.75</v>
       </c>
       <c r="D526">
-        <v>2666.56478480739</v>
+        <v>2666.7195882997999</v>
       </c>
       <c r="E526">
         <v>130.46378519162477</v>
@@ -14394,7 +14412,7 @@
         <v>81339.19</v>
       </c>
       <c r="D527">
-        <v>2620.5765563426598</v>
+        <v>2620.6928805780399</v>
       </c>
       <c r="E527">
         <v>130.55413121856733</v>
@@ -14417,7 +14435,7 @@
         <v>82008.69</v>
       </c>
       <c r="D528">
-        <v>2599.40268389531</v>
+        <v>2599.6951869702598</v>
       </c>
       <c r="E528">
         <v>131.77102810417074</v>
@@ -14440,7 +14458,7 @@
         <v>81730.81</v>
       </c>
       <c r="D529">
-        <v>2563.6928072875698</v>
+        <v>2563.6879177312098</v>
       </c>
       <c r="E529">
         <v>131.96378721102226</v>
@@ -14463,7 +14481,7 @@
         <v>82221.88</v>
       </c>
       <c r="D530">
-        <v>2560.4117340228199</v>
+        <v>2560.4027568052602</v>
       </c>
       <c r="E530">
         <v>132.47125094422424</v>
@@ -14486,7 +14504,7 @@
         <v>82346.94</v>
       </c>
       <c r="D531">
-        <v>2527.88825001234</v>
+        <v>2527.15409101266</v>
       </c>
       <c r="E531">
         <v>132.93298644421094</v>
@@ -14509,7 +14527,7 @@
         <v>82167</v>
       </c>
       <c r="D532">
-        <v>2513.2154258932601</v>
+        <v>2513.1125381390598</v>
       </c>
       <c r="E532">
         <v>132.44750488403352</v>
@@ -14532,7 +14550,7 @@
         <v>81802.94</v>
       </c>
       <c r="D533">
-        <v>2518.9817477821198</v>
+        <v>2518.9301776244401</v>
       </c>
       <c r="E533">
         <v>133.15785976208238</v>
@@ -14555,7 +14573,7 @@
         <v>81545.69</v>
       </c>
       <c r="D534">
-        <v>2511.4106567240801</v>
+        <v>2511.4218101169899</v>
       </c>
       <c r="E534">
         <v>132.90321082650064</v>
@@ -14578,7 +14596,7 @@
         <v>82230</v>
       </c>
       <c r="D535">
-        <v>2500.44271864957</v>
+        <v>2500.3222517612999</v>
       </c>
       <c r="E535">
         <v>132.70481133397854</v>
@@ -14601,7 +14619,7 @@
         <v>82667.88</v>
       </c>
       <c r="D536">
-        <v>2510.97528983858</v>
+        <v>2511.0237465700402</v>
       </c>
       <c r="E536">
         <v>133.07972091568664</v>
@@ -14624,10 +14642,10 @@
         <v>83433.63</v>
       </c>
       <c r="D537">
-        <v>2514.0158547825499</v>
+        <v>2514.3538294405698</v>
       </c>
       <c r="E537">
-        <v>133.65810791536416</v>
+        <v>133.65067677033733</v>
       </c>
       <c r="F537">
         <v>104.03270000000001</v>
@@ -14647,10 +14665,10 @@
         <v>83363.75</v>
       </c>
       <c r="D538">
-        <v>2509.3779916499998</v>
+        <v>2509.6973736965001</v>
       </c>
       <c r="E538">
-        <v>133.16905584985594</v>
+        <v>133.159422977715</v>
       </c>
       <c r="F538">
         <v>104.10039999999999</v>
@@ -14670,10 +14688,10 @@
         <v>84478.31</v>
       </c>
       <c r="D539">
-        <v>2520.7949003519702</v>
+        <v>2520.9949441613398</v>
       </c>
       <c r="E539">
-        <v>134.09423413483421</v>
+        <v>134.08243461507712</v>
       </c>
       <c r="F539">
         <v>103.98560000000001</v>
@@ -14693,10 +14711,10 @@
         <v>84611.5</v>
       </c>
       <c r="D540">
-        <v>2545.0477435939301</v>
+        <v>2545.40152890031</v>
       </c>
       <c r="E540">
-        <v>133.49283236360796</v>
+        <v>133.49864356080025</v>
       </c>
       <c r="F540">
         <v>104.0681</v>
@@ -14716,10 +14734,10 @@
         <v>84371.69</v>
       </c>
       <c r="D541">
-        <v>2557.18207885534</v>
+        <v>2557.38410609017</v>
       </c>
       <c r="E541">
-        <v>133.61733628620041</v>
+        <v>133.6238541456282</v>
       </c>
       <c r="F541">
         <v>104.0936</v>
@@ -14739,10 +14757,10 @@
         <v>82888.69</v>
       </c>
       <c r="D542">
-        <v>2542.1292392359401</v>
+        <v>2542.4084704851798</v>
       </c>
       <c r="E542">
-        <v>133.55832118988386</v>
+        <v>133.56866403399539</v>
       </c>
       <c r="F542">
         <v>103.4021</v>
@@ -14762,10 +14780,10 @@
         <v>82603.75</v>
       </c>
       <c r="D543">
-        <v>2530.9564884326101</v>
+        <v>2528.7506035004499</v>
       </c>
       <c r="E543">
-        <v>133.46484840479354</v>
+        <v>133.4937783333651</v>
       </c>
       <c r="F543">
         <v>102.83710000000001</v>
@@ -14785,10 +14803,10 @@
         <v>82528.69</v>
       </c>
       <c r="D544">
-        <v>2534.6713185569602</v>
+        <v>2534.9435178513299</v>
       </c>
       <c r="E544">
-        <v>134.23810593869791</v>
+        <v>134.26612326684631</v>
       </c>
       <c r="F544">
         <v>102.87569999999999</v>
@@ -14808,10 +14826,10 @@
         <v>82299.13</v>
       </c>
       <c r="D545">
-        <v>2518.5565867188998</v>
+        <v>2518.6259217316201</v>
       </c>
       <c r="E545">
-        <v>134.14139134314763</v>
+        <v>134.17591478155919</v>
       </c>
       <c r="F545">
         <v>102.274</v>
@@ -14831,10 +14849,10 @@
         <v>81535.63</v>
       </c>
       <c r="D546">
-        <v>2519.9754944089</v>
+        <v>2520.0307032939299</v>
       </c>
       <c r="E546">
-        <v>134.23909457870354</v>
+        <v>134.25153176848161</v>
       </c>
       <c r="F546">
         <v>102.392</v>
@@ -14854,10 +14872,10 @@
         <v>81712.81</v>
       </c>
       <c r="D547">
-        <v>2523.85628289755</v>
+        <v>2523.7129935090402</v>
       </c>
       <c r="E547">
-        <v>133.42403785544923</v>
+        <v>133.45443223898036</v>
       </c>
       <c r="F547">
         <v>102.4375</v>
@@ -14877,10 +14895,10 @@
         <v>81218.559999999998</v>
       </c>
       <c r="D548">
-        <v>2493.7056923570799</v>
+        <v>2493.88303602616</v>
       </c>
       <c r="E548">
-        <v>133.59534762851786</v>
+        <v>133.61623976098895</v>
       </c>
       <c r="F548">
         <v>101.9408</v>
@@ -14900,10 +14918,10 @@
         <v>82287.25</v>
       </c>
       <c r="D549">
-        <v>2510.99227651398</v>
+        <v>2511.34629801149</v>
       </c>
       <c r="E549">
-        <v>133.63061603917691</v>
+        <v>133.64469860722178</v>
       </c>
       <c r="F549">
         <v>102.639</v>
@@ -14923,10 +14941,10 @@
         <v>80615.25</v>
       </c>
       <c r="D550">
-        <v>2505.3077532350599</v>
+        <v>2505.83602086171</v>
       </c>
       <c r="E550">
-        <v>133.46455882413565</v>
+        <v>133.46851801539395</v>
       </c>
       <c r="F550">
         <v>102.29170000000001</v>
@@ -14946,10 +14964,10 @@
         <v>82476.88</v>
       </c>
       <c r="D551">
-        <v>2504.3446118602801</v>
+        <v>2504.6372635123098</v>
       </c>
       <c r="E551">
-        <v>133.6563763137313</v>
+        <v>133.66177641528549</v>
       </c>
       <c r="F551">
         <v>101.4281</v>
@@ -14969,10 +14987,10 @@
         <v>83394.880000000005</v>
       </c>
       <c r="D552">
-        <v>2500.5983722259398</v>
+        <v>2501.18696193917</v>
       </c>
       <c r="E552">
-        <v>133.93192151455256</v>
+        <v>133.94468599478679</v>
       </c>
       <c r="F552">
         <v>101.9372</v>
@@ -14992,10 +15010,10 @@
         <v>83462.69</v>
       </c>
       <c r="D553">
-        <v>2488.28197073926</v>
+        <v>2488.5340843451399</v>
       </c>
       <c r="E553">
-        <v>134.14632322772044</v>
+        <v>134.16612882337895</v>
       </c>
       <c r="F553">
         <v>101.7003</v>
@@ -15015,10 +15033,10 @@
         <v>82933.75</v>
       </c>
       <c r="D554">
-        <v>2482.87622166138</v>
+        <v>2483.26605328403</v>
       </c>
       <c r="E554">
-        <v>127.60414647932635</v>
+        <v>127.66912971222796</v>
       </c>
       <c r="F554">
         <v>101.0338</v>
@@ -15038,10 +15056,10 @@
         <v>82111</v>
       </c>
       <c r="D555">
-        <v>2472.5431200305102</v>
+        <v>2469.0190190308199</v>
       </c>
       <c r="E555">
-        <v>127.98893556293922</v>
+        <v>128.06744133285179</v>
       </c>
       <c r="F555">
         <v>101.37350000000001</v>
@@ -15061,10 +15079,10 @@
         <v>82233.81</v>
       </c>
       <c r="D556">
-        <v>2520.0310189298202</v>
+        <v>2520.4470066464301</v>
       </c>
       <c r="E556">
-        <v>127.65031301808182</v>
+        <v>127.7271957964585</v>
       </c>
       <c r="F556">
         <v>97.407799999999995</v>
@@ -15084,10 +15102,10 @@
         <v>82550.31</v>
       </c>
       <c r="D557">
-        <v>2595.7455999941699</v>
+        <v>2595.9488178127799</v>
       </c>
       <c r="E557">
-        <v>116.82282451701882</v>
+        <v>116.9094593718261</v>
       </c>
       <c r="F557">
         <v>84.561899999999994</v>
@@ -15107,10 +15125,10 @@
         <v>71432.13</v>
       </c>
       <c r="D558">
-        <v>2622.37368983952</v>
+        <v>2622.5404202851901</v>
       </c>
       <c r="E558">
-        <v>117.7913654348033</v>
+        <v>117.85233344680985</v>
       </c>
       <c r="F558">
         <v>85.960400000000007</v>
@@ -15130,10 +15148,10 @@
         <v>70177</v>
       </c>
       <c r="D559">
-        <v>2666.1406314311998</v>
+        <v>2666.1271918146899</v>
       </c>
       <c r="E559">
-        <v>123.27672498417164</v>
+        <v>123.35193015827606</v>
       </c>
       <c r="F559">
         <v>91.593400000000003</v>
@@ -15153,10 +15171,10 @@
         <v>71649.25</v>
       </c>
       <c r="D560">
-        <v>2665.7960372859702</v>
+        <v>2666.1825716124999</v>
       </c>
       <c r="E560">
-        <v>127.25618743223089</v>
+        <v>127.33643926328182</v>
       </c>
       <c r="F560">
         <v>95.025599999999997</v>
@@ -15176,10 +15194,10 @@
         <v>72757.13</v>
       </c>
       <c r="D561">
-        <v>2652.7937395025501</v>
+        <v>2653.1726518291298</v>
       </c>
       <c r="E561">
-        <v>128.96395051005075</v>
+        <v>129.04118020316363</v>
       </c>
       <c r="F561">
         <v>95.954899999999995</v>
@@ -15199,10 +15217,10 @@
         <v>72606.63</v>
       </c>
       <c r="D562">
-        <v>2647.6799222201998</v>
+        <v>2648.3966001787999</v>
       </c>
       <c r="E562">
-        <v>131.07514474364487</v>
+        <v>131.12876809185218</v>
       </c>
       <c r="F562">
         <v>95.966899999999995</v>
@@ -15222,10 +15240,10 @@
         <v>73182.31</v>
       </c>
       <c r="D563">
-        <v>2626.23035593851</v>
+        <v>2626.5034539885701</v>
       </c>
       <c r="E563">
-        <v>132.54404179522592</v>
+        <v>132.6055269121259</v>
       </c>
       <c r="F563">
         <v>96.739400000000003</v>
@@ -15245,10 +15263,10 @@
         <v>74978.94</v>
       </c>
       <c r="D564">
-        <v>2616.75250057942</v>
+        <v>2617.8544875023799</v>
       </c>
       <c r="E564">
-        <v>133.9465542762523</v>
+        <v>134.03304133938576</v>
       </c>
       <c r="F564">
         <v>97.081599999999995</v>
@@ -15268,10 +15286,10 @@
         <v>75718.880000000005</v>
       </c>
       <c r="D565">
-        <v>2618.9388266805299</v>
+        <v>2619.0167782380699</v>
       </c>
       <c r="E565">
-        <v>135.10112058040573</v>
+        <v>135.18145979699403</v>
       </c>
       <c r="F565">
         <v>98.363</v>
@@ -15291,16 +15309,16 @@
         <v>75922.5</v>
       </c>
       <c r="D566">
-        <v>2593.24048612874</v>
+        <v>2593.5412622465801</v>
       </c>
       <c r="E566">
-        <v>135.91735289756102</v>
+        <v>135.98689105914522</v>
       </c>
       <c r="F566">
         <v>98.882199999999997</v>
       </c>
       <c r="G566">
-        <v>262.63900000000001</v>
+        <v>262.68700000000001</v>
       </c>
     </row>
     <row r="567" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15314,16 +15332,16 @@
         <v>74006.13</v>
       </c>
       <c r="D567">
-        <v>2593.11692636932</v>
+        <v>2588.1386918196999</v>
       </c>
       <c r="E567">
-        <v>135.06210900907197</v>
+        <v>135.1392194227671</v>
       </c>
       <c r="F567">
         <v>95.614900000000006</v>
       </c>
       <c r="G567">
-        <v>263.57299999999998</v>
+        <v>263.57900000000001</v>
       </c>
     </row>
     <row r="568" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15337,16 +15355,16 @@
         <v>75878.559999999998</v>
       </c>
       <c r="D568">
-        <v>2557.8511170945999</v>
+        <v>2558.3961019178</v>
       </c>
       <c r="E568">
-        <v>136.13352295983407</v>
+        <v>136.22571270832398</v>
       </c>
       <c r="F568">
         <v>98.385599999999997</v>
       </c>
       <c r="G568">
-        <v>264.84699999999998</v>
+        <v>264.96100000000001</v>
       </c>
     </row>
     <row r="569" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15360,16 +15378,16 @@
         <v>75382.69</v>
       </c>
       <c r="D569">
-        <v>2513.0224528966601</v>
+        <v>2513.4557498447102</v>
       </c>
       <c r="E569">
-        <v>137.5598545210195</v>
+        <v>137.64564942626836</v>
       </c>
       <c r="F569">
         <v>98.558700000000002</v>
       </c>
       <c r="G569">
-        <v>266.625</v>
+        <v>266.61399999999998</v>
       </c>
     </row>
     <row r="570" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15383,16 +15401,16 @@
         <v>75885.06</v>
       </c>
       <c r="D570">
-        <v>2498.6159370580199</v>
+        <v>2498.9985361147301</v>
       </c>
       <c r="E570">
-        <v>136.0139445173086</v>
+        <v>136.05389989753658</v>
       </c>
       <c r="F570">
         <v>99.433300000000003</v>
       </c>
       <c r="G570">
-        <v>268.404</v>
+        <v>268.38299999999998</v>
       </c>
     </row>
     <row r="571" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15406,16 +15424,16 @@
         <v>76361</v>
       </c>
       <c r="D571">
-        <v>2456.7012534003902</v>
+        <v>2457.1845742417599</v>
       </c>
       <c r="E571">
-        <v>137.15169070819513</v>
+        <v>137.16216009258682</v>
       </c>
       <c r="F571">
         <v>99.798699999999997</v>
       </c>
       <c r="G571">
-        <v>270.70999999999998</v>
+        <v>270.654</v>
       </c>
     </row>
     <row r="572" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15429,16 +15447,16 @@
         <v>77642.559999999998</v>
       </c>
       <c r="D572">
-        <v>2439.3026917992902</v>
+        <v>2439.8379281799398</v>
       </c>
       <c r="E572">
-        <v>137.5284603615107</v>
+        <v>137.53122656301971</v>
       </c>
       <c r="F572">
         <v>100.25190000000001</v>
       </c>
       <c r="G572">
-        <v>271.96499999999997</v>
+        <v>271.90300000000002</v>
       </c>
     </row>
     <row r="573" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15452,16 +15470,16 @@
         <v>77234.06</v>
       </c>
       <c r="D573">
-        <v>2435.3486567517498</v>
+        <v>2435.7672276643202</v>
       </c>
       <c r="E573">
-        <v>136.9899519997887</v>
+        <v>136.99512698838896</v>
       </c>
       <c r="F573">
         <v>100.0437</v>
       </c>
       <c r="G573">
-        <v>272.75200000000001</v>
+        <v>272.67599999999999</v>
       </c>
     </row>
     <row r="574" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15475,16 +15493,16 @@
         <v>77634.94</v>
       </c>
       <c r="D574">
-        <v>2415.3830402840899</v>
+        <v>2416.2762991456102</v>
       </c>
       <c r="E574">
-        <v>136.35935956471712</v>
+        <v>136.31922406989943</v>
       </c>
       <c r="F574">
         <v>98.857900000000001</v>
       </c>
       <c r="G574">
-        <v>273.94200000000001</v>
+        <v>273.91000000000003</v>
       </c>
     </row>
     <row r="575" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15498,16 +15516,16 @@
         <v>78969.5</v>
       </c>
       <c r="D575">
-        <v>2411.2208902821799</v>
+        <v>2412.5375182978701</v>
       </c>
       <c r="E575">
-        <v>137.77323425500239</v>
+        <v>137.74665055013264</v>
       </c>
       <c r="F575">
         <v>100.1861</v>
       </c>
       <c r="G575">
-        <v>276.52800000000002</v>
+        <v>276.55</v>
       </c>
     </row>
     <row r="576" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15518,19 +15536,19 @@
         <v>79.150000000000006</v>
       </c>
       <c r="C576">
-        <v>79861.81</v>
+        <v>79827.69</v>
       </c>
       <c r="D576">
-        <v>2389.1205300521001</v>
+        <v>2391.79900422729</v>
       </c>
       <c r="E576">
-        <v>139.42524880931316</v>
+        <v>139.44267258599598</v>
       </c>
       <c r="F576">
         <v>100.86539999999999</v>
       </c>
       <c r="G576">
-        <v>278.82400000000001</v>
+        <v>278.91899999999998</v>
       </c>
     </row>
     <row r="577" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15541,19 +15559,19 @@
         <v>71.709999999999994</v>
       </c>
       <c r="C577">
-        <v>79392.31</v>
+        <v>79366.75</v>
       </c>
       <c r="D577">
-        <v>2364.1623880024999</v>
+        <v>2364.5694835723202</v>
       </c>
       <c r="E577">
-        <v>140.74117448039982</v>
+        <v>140.81205214436932</v>
       </c>
       <c r="F577">
         <v>100.57259999999999</v>
       </c>
       <c r="G577">
-        <v>280.80599999999998</v>
+        <v>280.84500000000003</v>
       </c>
     </row>
     <row r="578" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15564,19 +15582,19 @@
         <v>83.22</v>
       </c>
       <c r="C578">
-        <v>79552.38</v>
+        <v>79544.94</v>
       </c>
       <c r="D578">
-        <v>2330.06561961237</v>
+        <v>2330.7938082947699</v>
       </c>
       <c r="E578">
-        <v>141.17217050539756</v>
+        <v>141.11520203055548</v>
       </c>
       <c r="F578">
         <v>100.18559999999999</v>
       </c>
       <c r="G578">
-        <v>282.54199999999997</v>
+        <v>282.54300000000001</v>
       </c>
     </row>
     <row r="579" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15587,19 +15605,19 @@
         <v>91.64</v>
       </c>
       <c r="C579">
-        <v>80814.63</v>
+        <v>80818.31</v>
       </c>
       <c r="D579">
-        <v>2268.1202736477999</v>
+        <v>2263.58552786072</v>
       </c>
       <c r="E579">
-        <v>142.01203042127673</v>
+        <v>141.89557206449706</v>
       </c>
       <c r="F579">
         <v>100.8064</v>
       </c>
       <c r="G579">
-        <v>284.52499999999998</v>
+        <v>284.5</v>
       </c>
     </row>
     <row r="580" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15610,19 +15628,19 @@
         <v>108.5</v>
       </c>
       <c r="C580">
-        <v>80745.56</v>
+        <v>80746.75</v>
       </c>
       <c r="D580">
-        <v>2251.2438027541998</v>
+        <v>2252.0828825763301</v>
       </c>
       <c r="E580">
-        <v>141.386590814941</v>
+        <v>141.29459428789141</v>
       </c>
       <c r="F580">
         <v>101.3907</v>
       </c>
       <c r="G580">
-        <v>287.46699999999998</v>
+        <v>287.67399999999998</v>
       </c>
     </row>
     <row r="581" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15633,19 +15651,19 @@
         <v>101.78</v>
       </c>
       <c r="C581">
-        <v>79967.94</v>
+        <v>80001.94</v>
       </c>
       <c r="D581">
-        <v>2233.8785894019302</v>
+        <v>2235.7275641401602</v>
       </c>
       <c r="E581">
-        <v>139.70329988461529</v>
+        <v>139.63250258409872</v>
       </c>
       <c r="F581">
         <v>101.44</v>
       </c>
       <c r="G581">
-        <v>288.58199999999999</v>
+        <v>288.56099999999998</v>
       </c>
     </row>
     <row r="582" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15656,19 +15674,19 @@
         <v>109.55</v>
       </c>
       <c r="C582">
-        <v>79466.559999999998</v>
+        <v>79472.19</v>
       </c>
       <c r="D582">
-        <v>2187.8861448171901</v>
+        <v>2190.35679238791</v>
       </c>
       <c r="E582">
-        <v>140.5008531966717</v>
+        <v>140.35543238866498</v>
       </c>
       <c r="F582">
         <v>101.3335</v>
       </c>
       <c r="G582">
-        <v>291.29899999999998</v>
+        <v>291.298</v>
       </c>
     </row>
     <row r="583" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15679,19 +15697,19 @@
         <v>114.84</v>
       </c>
       <c r="C583">
-        <v>79717.19</v>
+        <v>79715.94</v>
       </c>
       <c r="D583">
-        <v>2164.0419250841601</v>
+        <v>2167.5525395701802</v>
       </c>
       <c r="E583">
-        <v>141.74164782447244</v>
+        <v>141.60750151547671</v>
       </c>
       <c r="F583">
         <v>101.018</v>
       </c>
       <c r="G583">
-        <v>295.072</v>
+        <v>294.95699999999999</v>
       </c>
     </row>
     <row r="584" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15702,19 +15720,19 @@
         <v>101.62</v>
       </c>
       <c r="C584">
-        <v>80628.13</v>
+        <v>80622.13</v>
       </c>
       <c r="D584">
-        <v>2142.63448609537</v>
+        <v>2143.3778313460898</v>
       </c>
       <c r="E584">
-        <v>141.45042270361822</v>
+        <v>141.33029180276199</v>
       </c>
       <c r="F584">
         <v>101.223</v>
       </c>
       <c r="G584">
-        <v>294.94</v>
+        <v>294.91300000000001</v>
       </c>
     </row>
     <row r="585" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15725,19 +15743,19 @@
         <v>93.67</v>
       </c>
       <c r="C585">
-        <v>81602.38</v>
+        <v>81595.13</v>
       </c>
       <c r="D585">
-        <v>2116.2039177888801</v>
+        <v>2117.96608194485</v>
       </c>
       <c r="E585">
-        <v>142.12083313138905</v>
+        <v>141.96568860854504</v>
       </c>
       <c r="F585">
         <v>101.0963</v>
       </c>
       <c r="G585">
-        <v>295.16199999999998</v>
+        <v>295.09699999999998</v>
       </c>
     </row>
     <row r="586" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15748,19 +15766,19 @@
         <v>84.26</v>
       </c>
       <c r="C586">
-        <v>82145.38</v>
+        <v>82137.94</v>
       </c>
       <c r="D586">
-        <v>2109.4059777068101</v>
+        <v>2112.2785716127501</v>
       </c>
       <c r="E586">
-        <v>142.72015775242571</v>
+        <v>142.55112807576546</v>
       </c>
       <c r="F586">
         <v>101.29179999999999</v>
       </c>
       <c r="G586">
-        <v>296.42099999999999</v>
+        <v>296.34899999999999</v>
       </c>
     </row>
     <row r="587" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15771,19 +15789,19 @@
         <v>87.55</v>
       </c>
       <c r="C587">
-        <v>82232.94</v>
+        <v>82226.559999999998</v>
       </c>
       <c r="D587">
-        <v>2075.10605030643</v>
+        <v>2076.1785042356501</v>
       </c>
       <c r="E587">
-        <v>141.99145145593877</v>
+        <v>141.80588567412346</v>
       </c>
       <c r="F587">
         <v>101.2529</v>
       </c>
       <c r="G587">
-        <v>297.97899999999998</v>
+        <v>298.00700000000001</v>
       </c>
     </row>
     <row r="588" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15794,19 +15812,19 @@
         <v>84.37</v>
       </c>
       <c r="C588">
-        <v>82561.13</v>
+        <v>82544.63</v>
       </c>
       <c r="D588">
-        <v>2007.2802218470999</v>
+        <v>2010.9412406163201</v>
       </c>
       <c r="E588">
-        <v>141.7819758335674</v>
+        <v>141.61984042213524</v>
       </c>
       <c r="F588">
         <v>100.9552</v>
       </c>
       <c r="G588">
-        <v>298.70800000000003</v>
+        <v>298.786</v>
       </c>
     </row>
     <row r="589" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15817,19 +15835,19 @@
         <v>76.44</v>
       </c>
       <c r="C589">
-        <v>81944.38</v>
+        <v>81927.88</v>
       </c>
       <c r="D589">
-        <v>2033.5934004471801</v>
+        <v>2034.1256771262399</v>
       </c>
       <c r="E589">
-        <v>141.11956260026543</v>
+        <v>140.93961230073265</v>
       </c>
       <c r="F589">
         <v>99.766400000000004</v>
       </c>
       <c r="G589">
-        <v>298.80799999999999</v>
+        <v>298.83199999999999</v>
       </c>
     </row>
     <row r="590" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15840,19 +15858,19 @@
         <v>78.12</v>
       </c>
       <c r="C590">
-        <v>82124.56</v>
+        <v>82091.56</v>
       </c>
       <c r="D590">
-        <v>2068.0681740446998</v>
+        <v>2067.1462221632901</v>
       </c>
       <c r="E590">
-        <v>141.62529271196013</v>
+        <v>141.45516232434346</v>
       </c>
       <c r="F590">
         <v>100.505</v>
       </c>
       <c r="G590">
-        <v>300.45600000000002</v>
+        <v>300.42</v>
       </c>
     </row>
     <row r="591" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15863,19 +15881,19 @@
         <v>76.83</v>
       </c>
       <c r="C591">
-        <v>82773.94</v>
+        <v>82741.63</v>
       </c>
       <c r="D591">
-        <v>2027.42833162785</v>
+        <v>2021.8132338079399</v>
       </c>
       <c r="E591">
-        <v>142.42784692897087</v>
+        <v>142.24732815523618</v>
       </c>
       <c r="F591">
         <v>100.6416</v>
       </c>
       <c r="G591">
-        <v>301.476</v>
+        <v>301.45</v>
       </c>
     </row>
     <row r="592" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15886,19 +15904,19 @@
         <v>73.28</v>
       </c>
       <c r="C592">
-        <v>82731.56</v>
+        <v>82699.63</v>
       </c>
       <c r="D592">
-        <v>2016.4754738101201</v>
+        <v>2017.5955506360201</v>
       </c>
       <c r="E592">
-        <v>142.57275415587222</v>
+        <v>142.50489486501837</v>
       </c>
       <c r="F592">
         <v>101.0205</v>
       </c>
       <c r="G592">
-        <v>301.64299999999997</v>
+        <v>301.82100000000003</v>
       </c>
     </row>
     <row r="593" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15909,19 +15927,19 @@
         <v>79.45</v>
       </c>
       <c r="C593">
-        <v>82150.13</v>
+        <v>82114.81</v>
       </c>
       <c r="D593">
-        <v>1984.1730935616799</v>
+        <v>1985.97384727553</v>
       </c>
       <c r="E593">
-        <v>141.62547728660985</v>
+        <v>141.50964977288419</v>
       </c>
       <c r="F593">
         <v>101.253</v>
       </c>
       <c r="G593">
-        <v>302.858</v>
+        <v>302.84500000000003</v>
       </c>
     </row>
     <row r="594" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15932,19 +15950,19 @@
         <v>71.58</v>
       </c>
       <c r="C594">
-        <v>81381.88</v>
+        <v>81346.44</v>
       </c>
       <c r="D594">
-        <v>1976.5705529218999</v>
+        <v>1979.3665705262199</v>
       </c>
       <c r="E594">
-        <v>142.44571945194784</v>
+        <v>142.3039535870723</v>
       </c>
       <c r="F594">
         <v>100.9286</v>
       </c>
       <c r="G594">
-        <v>303.31599999999997</v>
+        <v>303.334</v>
       </c>
     </row>
     <row r="595" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15955,19 +15973,19 @@
         <v>70.25</v>
       </c>
       <c r="C595">
-        <v>81978.25</v>
+        <v>81940.5</v>
       </c>
       <c r="D595">
-        <v>1975.55461678082</v>
+        <v>1980.1193524471</v>
       </c>
       <c r="E595">
-        <v>143.01742636471837</v>
+        <v>142.90640034148012</v>
       </c>
       <c r="F595">
         <v>100.11960000000001</v>
       </c>
       <c r="G595">
-        <v>304.09899999999999</v>
+        <v>304.01400000000001</v>
       </c>
     </row>
     <row r="596" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -15978,19 +15996,19 @@
         <v>76.069999999999993</v>
       </c>
       <c r="C596">
-        <v>81250.94</v>
+        <v>81210.94</v>
       </c>
       <c r="D596">
-        <v>1964.0541987629799</v>
+        <v>1964.73899156887</v>
       </c>
       <c r="E596">
-        <v>142.56849455773181</v>
+        <v>142.40442573493118</v>
       </c>
       <c r="F596">
         <v>100.9067</v>
       </c>
       <c r="G596">
-        <v>304.61500000000001</v>
+        <v>304.60899999999998</v>
       </c>
     </row>
     <row r="597" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16001,19 +16019,19 @@
         <v>81.39</v>
       </c>
       <c r="C597">
-        <v>80783.94</v>
+        <v>80762.69</v>
       </c>
       <c r="D597">
-        <v>1953.05309645432</v>
+        <v>1953.83062718582</v>
       </c>
       <c r="E597">
-        <v>143.16084305625412</v>
+        <v>143.01127915189505</v>
       </c>
       <c r="F597">
         <v>100.83929999999999</v>
       </c>
       <c r="G597">
-        <v>306.13799999999998</v>
+        <v>306.08199999999999</v>
       </c>
     </row>
     <row r="598" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16024,19 +16042,19 @@
         <v>89.43</v>
       </c>
       <c r="C598">
-        <v>81745.56</v>
+        <v>81724.31</v>
       </c>
       <c r="D598">
-        <v>1942.60094014728</v>
+        <v>1946.02322556232</v>
       </c>
       <c r="E598">
-        <v>143.4198416198395</v>
+        <v>143.35150642794963</v>
       </c>
       <c r="F598">
         <v>101.0211</v>
       </c>
       <c r="G598">
-        <v>307.37400000000002</v>
+        <v>307.27600000000001</v>
       </c>
     </row>
     <row r="599" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16047,19 +16065,19 @@
         <v>85.64</v>
       </c>
       <c r="C599">
-        <v>82099.5</v>
+        <v>82078.25</v>
       </c>
       <c r="D599">
-        <v>1944.4009091530399</v>
+        <v>1945.5176154021301</v>
       </c>
       <c r="E599">
-        <v>143.66440021969402</v>
+        <v>143.52873551435749</v>
       </c>
       <c r="F599">
         <v>100.4689</v>
       </c>
       <c r="G599">
-        <v>307.65300000000002</v>
+        <v>307.69600000000003</v>
       </c>
     </row>
     <row r="600" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16070,19 +16088,19 @@
         <v>77.69</v>
       </c>
       <c r="C600">
-        <v>82915.19</v>
+        <v>82893.69</v>
       </c>
       <c r="D600">
-        <v>1967.1396906284699</v>
+        <v>1970.9590953454499</v>
       </c>
       <c r="E600">
-        <v>144.11589703797998</v>
+        <v>144.01491438554649</v>
       </c>
       <c r="F600">
         <v>100.8639</v>
       </c>
       <c r="G600">
-        <v>308.08699999999999</v>
+        <v>308.14800000000002</v>
       </c>
     </row>
     <row r="601" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16093,19 +16111,19 @@
         <v>71.900000000000006</v>
       </c>
       <c r="C601">
-        <v>83215.75</v>
+        <v>83199.75</v>
       </c>
       <c r="D601">
-        <v>1962.2275395627501</v>
+        <v>1962.2337548333501</v>
       </c>
       <c r="E601">
-        <v>144.25923961837609</v>
+        <v>144.06551042465961</v>
       </c>
       <c r="F601">
         <v>100.6031</v>
       </c>
       <c r="G601">
-        <v>308.73500000000001</v>
+        <v>308.74099999999999</v>
       </c>
     </row>
     <row r="602" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16116,19 +16134,19 @@
         <v>74.150000000000006</v>
       </c>
       <c r="C602">
-        <v>81848.31</v>
+        <v>81780.69</v>
       </c>
       <c r="D602">
-        <v>1964.64964745515</v>
+        <v>1963.5157417365899</v>
       </c>
       <c r="E602">
-        <v>143.62968052067822</v>
+        <v>143.47766767134777</v>
       </c>
       <c r="F602">
         <v>99.222300000000004</v>
       </c>
       <c r="G602">
-        <v>309.79399999999998</v>
+        <v>309.69799999999998</v>
       </c>
     </row>
     <row r="603" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16139,19 +16157,19 @@
         <v>77.25</v>
       </c>
       <c r="C603">
-        <v>82540.88</v>
+        <v>82474.13</v>
       </c>
       <c r="D603">
-        <v>1982.83749666313</v>
+        <v>1978.3592108456901</v>
       </c>
       <c r="E603">
-        <v>144.35412774356155</v>
+        <v>144.22185649110688</v>
       </c>
       <c r="F603">
         <v>100.285</v>
       </c>
       <c r="G603">
-        <v>311.02199999999999</v>
+        <v>310.96699999999998</v>
       </c>
     </row>
     <row r="604" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16162,19 +16180,19 @@
         <v>81.28</v>
       </c>
       <c r="C604">
-        <v>82978.38</v>
+        <v>82884.88</v>
       </c>
       <c r="D604">
-        <v>1967.5023347103199</v>
+        <v>1967.7881871773</v>
       </c>
       <c r="E604">
-        <v>143.93086891497251</v>
+        <v>143.90923674577942</v>
       </c>
       <c r="F604">
         <v>100.4575</v>
       </c>
       <c r="G604">
-        <v>312.10700000000003</v>
+        <v>312.34500000000003</v>
       </c>
     </row>
     <row r="605" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16185,19 +16203,19 @@
         <v>85.35</v>
       </c>
       <c r="C605">
-        <v>82433.440000000002</v>
+        <v>82351</v>
       </c>
       <c r="D605">
-        <v>1994.29329509222</v>
+        <v>1995.1211427619201</v>
       </c>
       <c r="E605">
-        <v>144.53767445694857</v>
+        <v>144.50524604530958</v>
       </c>
       <c r="F605">
         <v>100.24339999999999</v>
       </c>
       <c r="G605">
-        <v>313.01600000000002</v>
+        <v>313.02300000000002</v>
       </c>
     </row>
     <row r="606" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16208,19 +16226,19 @@
         <v>80.02</v>
       </c>
       <c r="C606">
-        <v>81733.06</v>
+        <v>81640.38</v>
       </c>
       <c r="D606">
-        <v>1987.8741124256601</v>
+        <v>1991.10903594964</v>
       </c>
       <c r="E606">
-        <v>145.01253898824305</v>
+        <v>144.97598475286594</v>
       </c>
       <c r="F606">
         <v>100.863</v>
       </c>
       <c r="G606">
-        <v>313.14</v>
+        <v>313.17500000000001</v>
       </c>
     </row>
     <row r="607" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16231,19 +16249,19 @@
         <v>79.77</v>
       </c>
       <c r="C607">
-        <v>81435.19</v>
+        <v>81335.19</v>
       </c>
       <c r="D607">
-        <v>1989.8647843732999</v>
+        <v>1993.10966513932</v>
       </c>
       <c r="E607">
-        <v>145.13175820688275</v>
+        <v>144.98852611627615</v>
       </c>
       <c r="F607">
         <v>100.89400000000001</v>
       </c>
       <c r="G607">
-        <v>313.13099999999997</v>
+        <v>313.04399999999998</v>
       </c>
     </row>
     <row r="608" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16254,19 +16272,19 @@
         <v>81.8</v>
       </c>
       <c r="C608">
-        <v>81715.94</v>
+        <v>81635.81</v>
       </c>
       <c r="D608">
-        <v>1966.1400120822</v>
+        <v>1967.69407090138</v>
       </c>
       <c r="E608">
-        <v>145.48464989616389</v>
+        <v>145.34415303977144</v>
       </c>
       <c r="F608">
         <v>99.975700000000003</v>
       </c>
       <c r="G608">
-        <v>313.56599999999997</v>
+        <v>313.56900000000002</v>
       </c>
     </row>
     <row r="609" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16277,19 +16295,19 @@
         <v>76.680000000000007</v>
       </c>
       <c r="C609">
-        <v>81938.13</v>
+        <v>81854.94</v>
       </c>
       <c r="D609">
-        <v>1990.7882669386299</v>
+        <v>1991.63125800957</v>
       </c>
       <c r="E609">
-        <v>145.83398914726416</v>
+        <v>145.60409123922608</v>
       </c>
       <c r="F609">
         <v>100.43089999999999</v>
       </c>
       <c r="G609">
-        <v>314.13099999999997</v>
+        <v>314.06200000000001</v>
       </c>
     </row>
     <row r="610" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16300,19 +16318,19 @@
         <v>70.239999999999995</v>
       </c>
       <c r="C610">
-        <v>80860.38</v>
+        <v>80775.81</v>
       </c>
       <c r="D610">
-        <v>1996.5036865731199</v>
+        <v>2000.7953105434899</v>
       </c>
       <c r="E610">
-        <v>145.7453498293882</v>
+        <v>145.61711612476154</v>
       </c>
       <c r="F610">
         <v>99.808400000000006</v>
       </c>
       <c r="G610">
-        <v>314.851</v>
+        <v>314.73200000000003</v>
       </c>
     </row>
     <row r="611" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16323,19 +16341,19 @@
         <v>71.989999999999995</v>
       </c>
       <c r="C611">
-        <v>82023.56</v>
+        <v>81926.13</v>
       </c>
       <c r="D611">
-        <v>2004.88290849129</v>
+        <v>2004.85323222442</v>
       </c>
       <c r="E611">
-        <v>146.55848767053618</v>
+        <v>146.38329320972682</v>
       </c>
       <c r="F611">
         <v>99.469499999999996</v>
       </c>
       <c r="G611">
-        <v>315.56400000000002</v>
+        <v>315.63099999999997</v>
       </c>
     </row>
     <row r="612" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16346,19 +16364,19 @@
         <v>69.95</v>
       </c>
       <c r="C612">
-        <v>82238.38</v>
+        <v>82133.88</v>
       </c>
       <c r="D612">
-        <v>1991.36901132097</v>
+        <v>1995.1591679421199</v>
       </c>
       <c r="E612">
-        <v>146.56452763467027</v>
+        <v>146.43996866414332</v>
       </c>
       <c r="F612">
         <v>99.292500000000004</v>
       </c>
       <c r="G612">
-        <v>316.44900000000001</v>
+        <v>316.52800000000002</v>
       </c>
     </row>
     <row r="613" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16369,19 +16387,19 @@
         <v>70.12</v>
       </c>
       <c r="C613">
-        <v>82646.5</v>
+        <v>82557.88</v>
       </c>
       <c r="D613">
-        <v>2005.6491404523999</v>
+        <v>2004.7099317212801</v>
       </c>
       <c r="E613">
-        <v>147.65935784377464</v>
+        <v>147.55848999353427</v>
       </c>
       <c r="F613">
         <v>100.32729999999999</v>
       </c>
       <c r="G613">
-        <v>317.60300000000001</v>
+        <v>317.60399999999998</v>
       </c>
     </row>
     <row r="614" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16392,19 +16410,19 @@
         <v>75.739999999999995</v>
       </c>
       <c r="C614">
-        <v>82376.75</v>
+        <v>82150.31</v>
       </c>
       <c r="D614">
-        <v>2019.5848073862101</v>
+        <v>2015.8714990759499</v>
       </c>
       <c r="E614">
-        <v>147.22694372372359</v>
+        <v>107.084680646179</v>
       </c>
       <c r="F614">
         <v>100.0647</v>
       </c>
       <c r="G614">
-        <v>319.08600000000001</v>
+        <v>318.96100000000001</v>
       </c>
     </row>
     <row r="615" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16415,19 +16433,19 @@
         <v>71.53</v>
       </c>
       <c r="C615">
-        <v>82666.44</v>
+        <v>82418.38</v>
       </c>
       <c r="D615">
-        <v>2003.4907284979699</v>
+        <v>1996.0877065123</v>
       </c>
       <c r="E615">
-        <v>148.47042263320535</v>
+        <v>107.966246701709</v>
       </c>
       <c r="F615">
         <v>101.0993</v>
       </c>
       <c r="G615">
-        <v>319.77499999999998</v>
+        <v>319.67899999999997</v>
       </c>
     </row>
     <row r="616" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16438,19 +16456,19 @@
         <v>68.239999999999995</v>
       </c>
       <c r="C616">
-        <v>83778.75</v>
+        <v>83540.94</v>
       </c>
       <c r="D616">
-        <v>2004.9992607783799</v>
+        <v>2001.65554631336</v>
       </c>
       <c r="E616">
-        <v>149.08727424840274</v>
+        <v>108.36047415102099</v>
       </c>
       <c r="F616">
         <v>101.04040000000001</v>
       </c>
       <c r="G616">
-        <v>319.61500000000001</v>
+        <v>319.78500000000003</v>
       </c>
     </row>
     <row r="617" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16461,19 +16479,19 @@
         <v>63.54</v>
       </c>
       <c r="C617">
-        <v>83227.94</v>
+        <v>82978.25</v>
       </c>
       <c r="D617">
-        <v>1986.8172638992801</v>
+        <v>1985.73278300633</v>
       </c>
       <c r="E617">
-        <v>148.94509250450278</v>
+        <v>108.23326716438</v>
       </c>
       <c r="F617">
         <v>101.1279</v>
       </c>
       <c r="G617">
-        <v>320.32100000000003</v>
+        <v>320.30200000000002</v>
       </c>
     </row>
     <row r="618" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16484,19 +16502,19 @@
         <v>62.17</v>
       </c>
       <c r="C618">
-        <v>83313.13</v>
+        <v>83068.13</v>
       </c>
       <c r="D618">
-        <v>1992.58894702619</v>
+        <v>1993.5968582944499</v>
       </c>
       <c r="E618">
-        <v>149.35412984112781</v>
+        <v>108.601629715882</v>
       </c>
       <c r="F618">
-        <v>100.9773</v>
+        <v>100.96550000000001</v>
       </c>
       <c r="G618">
-        <v>320.58</v>
+        <v>320.62</v>
       </c>
     </row>
     <row r="619" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -16507,19 +16525,157 @@
         <v>68.17</v>
       </c>
       <c r="C619">
-        <v>84405.13</v>
+        <v>84156.69</v>
       </c>
       <c r="D619">
-        <v>1984.17213663537</v>
+        <v>1988.6415974287499</v>
       </c>
       <c r="E619">
-        <v>149.72210402155815</v>
+        <v>108.959154727925</v>
       </c>
       <c r="F619">
-        <v>101.428</v>
+        <v>101.4785</v>
       </c>
       <c r="G619">
-        <v>321.5</v>
+        <v>321.435</v>
+      </c>
+    </row>
+    <row r="620" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A620" t="s">
+        <v>625</v>
+      </c>
+      <c r="B620">
+        <v>68.39</v>
+      </c>
+      <c r="C620">
+        <v>84562.44</v>
+      </c>
+      <c r="D620">
+        <v>2009.82017959069</v>
+      </c>
+      <c r="E620">
+        <v>109.165462336365</v>
+      </c>
+      <c r="F620">
+        <v>101.89400000000001</v>
+      </c>
+      <c r="G620">
+        <v>322.16899999999998</v>
+      </c>
+    </row>
+    <row r="621" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A621" t="s">
+        <v>626</v>
+      </c>
+      <c r="B621">
+        <v>64.86</v>
+      </c>
+      <c r="C621">
+        <v>85042.75</v>
+      </c>
+      <c r="D621">
+        <v>2026.4874779014499</v>
+      </c>
+      <c r="E621">
+        <v>108.886271701712</v>
+      </c>
+      <c r="F621">
+        <v>101.6247</v>
+      </c>
+      <c r="G621">
+        <v>323.291</v>
+      </c>
+    </row>
+    <row r="622" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A622" t="s">
+        <v>627</v>
+      </c>
+      <c r="B622">
+        <v>63.96</v>
+      </c>
+      <c r="C622">
+        <v>86164.75</v>
+      </c>
+      <c r="D622">
+        <v>2018.8592186267001</v>
+      </c>
+      <c r="E622">
+        <v>109.905439643118</v>
+      </c>
+      <c r="F622">
+        <v>101.66800000000001</v>
+      </c>
+      <c r="G622">
+        <v>324.245</v>
+      </c>
+    </row>
+    <row r="623" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A623" t="s">
+        <v>628</v>
+      </c>
+      <c r="B623">
+        <v>60.89</v>
+      </c>
+      <c r="C623">
+        <v>86110.25</v>
+      </c>
+      <c r="D623">
+        <v>2024.90263173023</v>
+      </c>
+      <c r="E623">
+        <v>109.605428443696</v>
+      </c>
+      <c r="F623">
+        <v>101.2075</v>
+      </c>
+      <c r="G623">
+        <v>324.654</v>
+      </c>
+    </row>
+    <row r="624" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A624" t="s">
+        <v>629</v>
+      </c>
+      <c r="B624">
+        <v>60.06</v>
+      </c>
+      <c r="C624">
+        <v>86079.88</v>
+      </c>
+      <c r="D624">
+        <v>2011.2843671400799</v>
+      </c>
+      <c r="E624">
+        <v>109.942326464494</v>
+      </c>
+      <c r="F624">
+        <v>101.3605</v>
+      </c>
+      <c r="G624">
+        <v>325.06299999999999</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A625" t="s">
+        <v>630</v>
+      </c>
+      <c r="B625">
+        <v>57.97</v>
+      </c>
+      <c r="C625">
+        <v>85891.5</v>
+      </c>
+      <c r="D625">
+        <v>2001.77582591138</v>
+      </c>
+      <c r="E625">
+        <v>110.66823508944</v>
+      </c>
+      <c r="F625">
+        <v>101.6781</v>
+      </c>
+      <c r="G625">
+        <v>326.03100000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>